<commit_message>
Cadrage évolué : leviers de coûts + colonne Budget N+1 dans le P&L
- 01_Cadrage : ajout de 2 leviers de coûts (inflation charges externes,
  politique salariale) — le cadrage pilote désormais CA ET coûts
- 07_PnL : colonne Budget N+1 pilotée par le cadrage — produits & coûts
  directs scalent avec le CA moteur, personnel avec effectif × salaire,
  structure/impôts/D&A avec l'inflation
- Budget scénario Cadrage : CA 24,3 M€, EBITDA 16,9% (levier opérationnel) ;
  scénario Référence reproduit l'atterrissage (14,6%)
- 0 erreur, budget CA tie-out avec le moteur

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_CA_v3.xlsx
+++ b/eduservices/EDUSERVICES_Modele_CA_v3.xlsx
@@ -83,7 +83,7 @@
       <color rgb="000000FF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -115,6 +115,11 @@
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF3EA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -142,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -292,7 +297,13 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -775,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:M24"/>
+  <dimension ref="B1:M26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1348,10 +1359,31 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="32" t="inlineStr">
-        <is>
-          <t>Astuce : choisir « Référence » remet tous les leviers à 0 → le modèle reproduit l'atterrissage.</t>
-        </is>
+      <c r="B19" s="27" t="inlineStr">
+        <is>
+          <t>Inflation des charges externes (→ coûts)</t>
+        </is>
+      </c>
+      <c r="C19" s="28" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D19" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F19" s="30" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="G19" s="30" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H19" s="31">
+        <f>INDEX(D19:G19,MATCH($D$3,$D$13:$G$13,0))</f>
+        <v/>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
@@ -1371,18 +1403,33 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>③ Constantes de référence (scénarisables)</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n"/>
-      <c r="H20" s="4" t="n"/>
+    <row r="20">
+      <c r="B20" s="27" t="inlineStr">
+        <is>
+          <t>Politique salariale (→ personnel)</t>
+        </is>
+      </c>
+      <c r="C20" s="28" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D20" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="30" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F20" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G20" s="30" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H20" s="31">
+        <f>INDEX(D20:G20,MATCH($D$3,$D$13:$G$13,0))</f>
+        <v/>
+      </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
           <t>Tunon</t>
@@ -1402,135 +1449,155 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="32" t="inlineStr">
+        <is>
+          <t>Leviers 1-5 → CA (moteur) · leviers 6-7 → coûts (P&amp;L Budget N+1). « Référence » remet tout à 0 = atterrissage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>③ Constantes de référence (scénarisables)</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>Paramètre</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C23" s="10" t="inlineStr">
         <is>
           <t>Unité</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
+      <c r="D23" s="10" t="inlineStr">
         <is>
           <t>Référence</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>Cadrage</t>
         </is>
       </c>
-      <c r="F21" s="10" t="inlineStr">
+      <c r="F23" s="10" t="inlineStr">
         <is>
           <t>Optimiste</t>
         </is>
       </c>
-      <c r="G21" s="10" t="inlineStr">
+      <c r="G23" s="10" t="inlineStr">
         <is>
           <t>Prudent</t>
         </is>
       </c>
-      <c r="H21" s="10" t="inlineStr">
+      <c r="H23" s="10" t="inlineStr">
         <is>
           <t>ACTIF</t>
         </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="27" t="inlineStr">
-        <is>
-          <t>Rendement d'acquisition (part payante)</t>
-        </is>
-      </c>
-      <c r="C22" s="28" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="D22" s="33" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E22" s="19" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F22" s="19" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G22" s="19" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H22" s="34">
-        <f>INDEX(D22:G22,MATCH($D$3,$D$13:$G$13,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="27" t="inlineStr">
-        <is>
-          <t>Part organique des leads (hors budget)</t>
-        </is>
-      </c>
-      <c r="C23" s="28" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D23" s="29" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="E23" s="30" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F23" s="30" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G23" s="30" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H23" s="31">
-        <f>INDEX(D23:G23,MATCH($D$3,$D$13:$G$13,0))</f>
-        <v/>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="27" t="inlineStr">
         <is>
+          <t>Rendement d'acquisition (part payante)</t>
+        </is>
+      </c>
+      <c r="C24" s="28" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D24" s="33" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E24" s="19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F24" s="19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G24" s="19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H24" s="34">
+        <f>INDEX(D24:G24,MATCH($D$3,$D$13:$G$13,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="27" t="inlineStr">
+        <is>
+          <t>Part organique des leads (hors budget)</t>
+        </is>
+      </c>
+      <c r="C25" s="28" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D25" s="29" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E25" s="30" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F25" s="30" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G25" s="30" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H25" s="31">
+        <f>INDEX(D25:G25,MATCH($D$3,$D$13:$G$13,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="27" t="inlineStr">
+        <is>
           <t>Frais de dossier / nouvel inscrit</t>
         </is>
       </c>
-      <c r="C24" s="28" t="inlineStr">
+      <c r="C26" s="28" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="D24" s="35" t="n">
+      <c r="D26" s="35" t="n">
         <v>90</v>
       </c>
-      <c r="E24" s="36" t="n">
+      <c r="E26" s="36" t="n">
         <v>90</v>
       </c>
-      <c r="F24" s="36" t="n">
+      <c r="F26" s="36" t="n">
         <v>90</v>
       </c>
-      <c r="G24" s="36" t="n">
+      <c r="G26" s="36" t="n">
         <v>90</v>
       </c>
-      <c r="H24" s="37">
-        <f>INDEX(D24:G24,MATCH($D$3,$D$13:$G$13,0))</f>
+      <c r="H26" s="37">
+        <f>INDEX(D26:G26,MATCH($D$3,$D$13:$G$13,0))</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="J5:M5"/>
+    <mergeCell ref="B22:H22"/>
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B21:H21"/>
     <mergeCell ref="B12:H12"/>
     <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B19:H19"/>
-    <mergeCell ref="B20:H20"/>
+    <mergeCell ref="J5:M5"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="D3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -6114,7 +6181,7 @@
         <v/>
       </c>
       <c r="E5" s="41">
-        <f>'01_Cadrage'!$H$23</f>
+        <f>'01_Cadrage'!$H$25</f>
         <v/>
       </c>
       <c r="F5" s="24">
@@ -6137,7 +6204,7 @@
         <v/>
       </c>
       <c r="K5" s="22">
-        <f>G5*(J5/I5)^'01_Cadrage'!$H$22</f>
+        <f>G5*(J5/I5)^'01_Cadrage'!$H$24</f>
         <v/>
       </c>
       <c r="L5" s="22">
@@ -6169,7 +6236,7 @@
         <v/>
       </c>
       <c r="E6" s="41">
-        <f>'01_Cadrage'!$H$23</f>
+        <f>'01_Cadrage'!$H$25</f>
         <v/>
       </c>
       <c r="F6" s="24">
@@ -6192,7 +6259,7 @@
         <v/>
       </c>
       <c r="K6" s="22">
-        <f>G6*(J6/I6)^'01_Cadrage'!$H$22</f>
+        <f>G6*(J6/I6)^'01_Cadrage'!$H$24</f>
         <v/>
       </c>
       <c r="L6" s="22">
@@ -6224,7 +6291,7 @@
         <v/>
       </c>
       <c r="E7" s="41">
-        <f>'01_Cadrage'!$H$23</f>
+        <f>'01_Cadrage'!$H$25</f>
         <v/>
       </c>
       <c r="F7" s="24">
@@ -6247,7 +6314,7 @@
         <v/>
       </c>
       <c r="K7" s="22">
-        <f>G7*(J7/I7)^'01_Cadrage'!$H$22</f>
+        <f>G7*(J7/I7)^'01_Cadrage'!$H$24</f>
         <v/>
       </c>
       <c r="L7" s="22">
@@ -6279,7 +6346,7 @@
         <v/>
       </c>
       <c r="E8" s="41">
-        <f>'01_Cadrage'!$H$23</f>
+        <f>'01_Cadrage'!$H$25</f>
         <v/>
       </c>
       <c r="F8" s="24">
@@ -6302,7 +6369,7 @@
         <v/>
       </c>
       <c r="K8" s="22">
-        <f>G8*(J8/I8)^'01_Cadrage'!$H$22</f>
+        <f>G8*(J8/I8)^'01_Cadrage'!$H$24</f>
         <v/>
       </c>
       <c r="L8" s="22">
@@ -6334,7 +6401,7 @@
         <v/>
       </c>
       <c r="E9" s="41">
-        <f>'01_Cadrage'!$H$23</f>
+        <f>'01_Cadrage'!$H$25</f>
         <v/>
       </c>
       <c r="F9" s="24">
@@ -6357,7 +6424,7 @@
         <v/>
       </c>
       <c r="K9" s="22">
-        <f>G9*(J9/I9)^'01_Cadrage'!$H$22</f>
+        <f>G9*(J9/I9)^'01_Cadrage'!$H$24</f>
         <v/>
       </c>
       <c r="L9" s="22">
@@ -6389,7 +6456,7 @@
         <v/>
       </c>
       <c r="E10" s="41">
-        <f>'01_Cadrage'!$H$23</f>
+        <f>'01_Cadrage'!$H$25</f>
         <v/>
       </c>
       <c r="F10" s="24">
@@ -6412,7 +6479,7 @@
         <v/>
       </c>
       <c r="K10" s="22">
-        <f>G10*(J10/I10)^'01_Cadrage'!$H$22</f>
+        <f>G10*(J10/I10)^'01_Cadrage'!$H$24</f>
         <v/>
       </c>
       <c r="L10" s="22">
@@ -6444,7 +6511,7 @@
         <v/>
       </c>
       <c r="E11" s="41">
-        <f>'01_Cadrage'!$H$23</f>
+        <f>'01_Cadrage'!$H$25</f>
         <v/>
       </c>
       <c r="F11" s="24">
@@ -6467,7 +6534,7 @@
         <v/>
       </c>
       <c r="K11" s="22">
-        <f>G11*(J11/I11)^'01_Cadrage'!$H$22</f>
+        <f>G11*(J11/I11)^'01_Cadrage'!$H$24</f>
         <v/>
       </c>
       <c r="L11" s="22">
@@ -6499,7 +6566,7 @@
         <v/>
       </c>
       <c r="E12" s="41">
-        <f>'01_Cadrage'!$H$23</f>
+        <f>'01_Cadrage'!$H$25</f>
         <v/>
       </c>
       <c r="F12" s="24">
@@ -6522,7 +6589,7 @@
         <v/>
       </c>
       <c r="K12" s="22">
-        <f>G12*(J12/I12)^'01_Cadrage'!$H$22</f>
+        <f>G12*(J12/I12)^'01_Cadrage'!$H$24</f>
         <v/>
       </c>
       <c r="L12" s="22">
@@ -6554,7 +6621,7 @@
         <v/>
       </c>
       <c r="E13" s="41">
-        <f>'01_Cadrage'!$H$23</f>
+        <f>'01_Cadrage'!$H$25</f>
         <v/>
       </c>
       <c r="F13" s="24">
@@ -6577,7 +6644,7 @@
         <v/>
       </c>
       <c r="K13" s="22">
-        <f>G13*(J13/I13)^'01_Cadrage'!$H$22</f>
+        <f>G13*(J13/I13)^'01_Cadrage'!$H$24</f>
         <v/>
       </c>
       <c r="L13" s="22">
@@ -6609,7 +6676,7 @@
         <v/>
       </c>
       <c r="E14" s="41">
-        <f>'01_Cadrage'!$H$23</f>
+        <f>'01_Cadrage'!$H$25</f>
         <v/>
       </c>
       <c r="F14" s="24">
@@ -6632,7 +6699,7 @@
         <v/>
       </c>
       <c r="K14" s="22">
-        <f>G14*(J14/I14)^'01_Cadrage'!$H$22</f>
+        <f>G14*(J14/I14)^'01_Cadrage'!$H$24</f>
         <v/>
       </c>
       <c r="L14" s="22">
@@ -6664,7 +6731,7 @@
         <v/>
       </c>
       <c r="E15" s="41">
-        <f>'01_Cadrage'!$H$23</f>
+        <f>'01_Cadrage'!$H$25</f>
         <v/>
       </c>
       <c r="F15" s="24">
@@ -6687,7 +6754,7 @@
         <v/>
       </c>
       <c r="K15" s="22">
-        <f>G15*(J15/I15)^'01_Cadrage'!$H$22</f>
+        <f>G15*(J15/I15)^'01_Cadrage'!$H$24</f>
         <v/>
       </c>
       <c r="L15" s="22">
@@ -6719,7 +6786,7 @@
         <v/>
       </c>
       <c r="E16" s="41">
-        <f>'01_Cadrage'!$H$23</f>
+        <f>'01_Cadrage'!$H$25</f>
         <v/>
       </c>
       <c r="F16" s="24">
@@ -6742,7 +6809,7 @@
         <v/>
       </c>
       <c r="K16" s="22">
-        <f>G16*(J16/I16)^'01_Cadrage'!$H$22</f>
+        <f>G16*(J16/I16)^'01_Cadrage'!$H$24</f>
         <v/>
       </c>
       <c r="L16" s="22">
@@ -6774,7 +6841,7 @@
         <v/>
       </c>
       <c r="E17" s="41">
-        <f>'01_Cadrage'!$H$23</f>
+        <f>'01_Cadrage'!$H$25</f>
         <v/>
       </c>
       <c r="F17" s="24">
@@ -6797,7 +6864,7 @@
         <v/>
       </c>
       <c r="K17" s="22">
-        <f>G17*(J17/I17)^'01_Cadrage'!$H$22</f>
+        <f>G17*(J17/I17)^'01_Cadrage'!$H$24</f>
         <v/>
       </c>
       <c r="L17" s="22">
@@ -6829,7 +6896,7 @@
         <v/>
       </c>
       <c r="E18" s="41">
-        <f>'01_Cadrage'!$H$23</f>
+        <f>'01_Cadrage'!$H$25</f>
         <v/>
       </c>
       <c r="F18" s="24">
@@ -6852,7 +6919,7 @@
         <v/>
       </c>
       <c r="K18" s="22">
-        <f>G18*(J18/I18)^'01_Cadrage'!$H$22</f>
+        <f>G18*(J18/I18)^'01_Cadrage'!$H$24</f>
         <v/>
       </c>
       <c r="L18" s="22">
@@ -7161,7 +7228,7 @@
         <v/>
       </c>
       <c r="AA4" s="13">
-        <f>Y4*Z4+W4*'01_Cadrage'!$H$24</f>
+        <f>Y4*Z4+W4*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -7271,7 +7338,7 @@
         <v/>
       </c>
       <c r="AA5" s="13">
-        <f>Y5*Z5+W5*'01_Cadrage'!$H$24</f>
+        <f>Y5*Z5+W5*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -7381,7 +7448,7 @@
         <v/>
       </c>
       <c r="AA6" s="13">
-        <f>Y6*Z6+W6*'01_Cadrage'!$H$24</f>
+        <f>Y6*Z6+W6*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -7491,7 +7558,7 @@
         <v/>
       </c>
       <c r="AA7" s="13">
-        <f>Y7*Z7+W7*'01_Cadrage'!$H$24</f>
+        <f>Y7*Z7+W7*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -7601,7 +7668,7 @@
         <v/>
       </c>
       <c r="AA8" s="13">
-        <f>Y8*Z8+W8*'01_Cadrage'!$H$24</f>
+        <f>Y8*Z8+W8*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -7711,7 +7778,7 @@
         <v/>
       </c>
       <c r="AA9" s="13">
-        <f>Y9*Z9+W9*'01_Cadrage'!$H$24</f>
+        <f>Y9*Z9+W9*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -7821,7 +7888,7 @@
         <v/>
       </c>
       <c r="AA10" s="13">
-        <f>Y10*Z10+W10*'01_Cadrage'!$H$24</f>
+        <f>Y10*Z10+W10*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -7931,7 +7998,7 @@
         <v/>
       </c>
       <c r="AA11" s="13">
-        <f>Y11*Z11+W11*'01_Cadrage'!$H$24</f>
+        <f>Y11*Z11+W11*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -8041,7 +8108,7 @@
         <v/>
       </c>
       <c r="AA12" s="13">
-        <f>Y12*Z12+W12*'01_Cadrage'!$H$24</f>
+        <f>Y12*Z12+W12*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -8151,7 +8218,7 @@
         <v/>
       </c>
       <c r="AA13" s="13">
-        <f>Y13*Z13+W13*'01_Cadrage'!$H$24</f>
+        <f>Y13*Z13+W13*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -8261,7 +8328,7 @@
         <v/>
       </c>
       <c r="AA14" s="13">
-        <f>Y14*Z14+W14*'01_Cadrage'!$H$24</f>
+        <f>Y14*Z14+W14*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -8371,7 +8438,7 @@
         <v/>
       </c>
       <c r="AA15" s="13">
-        <f>Y15*Z15+W15*'01_Cadrage'!$H$24</f>
+        <f>Y15*Z15+W15*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -8481,7 +8548,7 @@
         <v/>
       </c>
       <c r="AA16" s="13">
-        <f>Y16*Z16+W16*'01_Cadrage'!$H$24</f>
+        <f>Y16*Z16+W16*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -8591,7 +8658,7 @@
         <v/>
       </c>
       <c r="AA17" s="13">
-        <f>Y17*Z17+W17*'01_Cadrage'!$H$24</f>
+        <f>Y17*Z17+W17*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -8701,7 +8768,7 @@
         <v/>
       </c>
       <c r="AA18" s="13">
-        <f>Y18*Z18+W18*'01_Cadrage'!$H$24</f>
+        <f>Y18*Z18+W18*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -8811,7 +8878,7 @@
         <v/>
       </c>
       <c r="AA19" s="13">
-        <f>Y19*Z19+W19*'01_Cadrage'!$H$24</f>
+        <f>Y19*Z19+W19*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -8921,7 +8988,7 @@
         <v/>
       </c>
       <c r="AA20" s="13">
-        <f>Y20*Z20+W20*'01_Cadrage'!$H$24</f>
+        <f>Y20*Z20+W20*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -9031,7 +9098,7 @@
         <v/>
       </c>
       <c r="AA21" s="13">
-        <f>Y21*Z21+W21*'01_Cadrage'!$H$24</f>
+        <f>Y21*Z21+W21*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -9141,7 +9208,7 @@
         <v/>
       </c>
       <c r="AA22" s="13">
-        <f>Y22*Z22+W22*'01_Cadrage'!$H$24</f>
+        <f>Y22*Z22+W22*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -9251,7 +9318,7 @@
         <v/>
       </c>
       <c r="AA23" s="13">
-        <f>Y23*Z23+W23*'01_Cadrage'!$H$24</f>
+        <f>Y23*Z23+W23*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -9361,7 +9428,7 @@
         <v/>
       </c>
       <c r="AA24" s="13">
-        <f>Y24*Z24+W24*'01_Cadrage'!$H$24</f>
+        <f>Y24*Z24+W24*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -9471,7 +9538,7 @@
         <v/>
       </c>
       <c r="AA25" s="13">
-        <f>Y25*Z25+W25*'01_Cadrage'!$H$24</f>
+        <f>Y25*Z25+W25*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -9581,7 +9648,7 @@
         <v/>
       </c>
       <c r="AA26" s="13">
-        <f>Y26*Z26+W26*'01_Cadrage'!$H$24</f>
+        <f>Y26*Z26+W26*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -9691,7 +9758,7 @@
         <v/>
       </c>
       <c r="AA27" s="13">
-        <f>Y27*Z27+W27*'01_Cadrage'!$H$24</f>
+        <f>Y27*Z27+W27*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -9801,7 +9868,7 @@
         <v/>
       </c>
       <c r="AA28" s="13">
-        <f>Y28*Z28+W28*'01_Cadrage'!$H$24</f>
+        <f>Y28*Z28+W28*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -9911,7 +9978,7 @@
         <v/>
       </c>
       <c r="AA29" s="13">
-        <f>Y29*Z29+W29*'01_Cadrage'!$H$24</f>
+        <f>Y29*Z29+W29*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -10021,7 +10088,7 @@
         <v/>
       </c>
       <c r="AA30" s="13">
-        <f>Y30*Z30+W30*'01_Cadrage'!$H$24</f>
+        <f>Y30*Z30+W30*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -10131,7 +10198,7 @@
         <v/>
       </c>
       <c r="AA31" s="13">
-        <f>Y31*Z31+W31*'01_Cadrage'!$H$24</f>
+        <f>Y31*Z31+W31*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -10241,7 +10308,7 @@
         <v/>
       </c>
       <c r="AA32" s="13">
-        <f>Y32*Z32+W32*'01_Cadrage'!$H$24</f>
+        <f>Y32*Z32+W32*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -10351,7 +10418,7 @@
         <v/>
       </c>
       <c r="AA33" s="13">
-        <f>Y33*Z33+W33*'01_Cadrage'!$H$24</f>
+        <f>Y33*Z33+W33*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -10461,7 +10528,7 @@
         <v/>
       </c>
       <c r="AA34" s="13">
-        <f>Y34*Z34+W34*'01_Cadrage'!$H$24</f>
+        <f>Y34*Z34+W34*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -10571,7 +10638,7 @@
         <v/>
       </c>
       <c r="AA35" s="13">
-        <f>Y35*Z35+W35*'01_Cadrage'!$H$24</f>
+        <f>Y35*Z35+W35*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -10681,7 +10748,7 @@
         <v/>
       </c>
       <c r="AA36" s="13">
-        <f>Y36*Z36+W36*'01_Cadrage'!$H$24</f>
+        <f>Y36*Z36+W36*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -10791,7 +10858,7 @@
         <v/>
       </c>
       <c r="AA37" s="13">
-        <f>Y37*Z37+W37*'01_Cadrage'!$H$24</f>
+        <f>Y37*Z37+W37*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -10901,7 +10968,7 @@
         <v/>
       </c>
       <c r="AA38" s="13">
-        <f>Y38*Z38+W38*'01_Cadrage'!$H$24</f>
+        <f>Y38*Z38+W38*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -11011,7 +11078,7 @@
         <v/>
       </c>
       <c r="AA39" s="13">
-        <f>Y39*Z39+W39*'01_Cadrage'!$H$24</f>
+        <f>Y39*Z39+W39*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -11121,7 +11188,7 @@
         <v/>
       </c>
       <c r="AA40" s="13">
-        <f>Y40*Z40+W40*'01_Cadrage'!$H$24</f>
+        <f>Y40*Z40+W40*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -11231,7 +11298,7 @@
         <v/>
       </c>
       <c r="AA41" s="13">
-        <f>Y41*Z41+W41*'01_Cadrage'!$H$24</f>
+        <f>Y41*Z41+W41*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -11341,7 +11408,7 @@
         <v/>
       </c>
       <c r="AA42" s="13">
-        <f>Y42*Z42+W42*'01_Cadrage'!$H$24</f>
+        <f>Y42*Z42+W42*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -11451,7 +11518,7 @@
         <v/>
       </c>
       <c r="AA43" s="13">
-        <f>Y43*Z43+W43*'01_Cadrage'!$H$24</f>
+        <f>Y43*Z43+W43*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -11561,7 +11628,7 @@
         <v/>
       </c>
       <c r="AA44" s="13">
-        <f>Y44*Z44+W44*'01_Cadrage'!$H$24</f>
+        <f>Y44*Z44+W44*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -11671,7 +11738,7 @@
         <v/>
       </c>
       <c r="AA45" s="13">
-        <f>Y45*Z45+W45*'01_Cadrage'!$H$24</f>
+        <f>Y45*Z45+W45*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -11781,7 +11848,7 @@
         <v/>
       </c>
       <c r="AA46" s="13">
-        <f>Y46*Z46+W46*'01_Cadrage'!$H$24</f>
+        <f>Y46*Z46+W46*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -11891,7 +11958,7 @@
         <v/>
       </c>
       <c r="AA47" s="13">
-        <f>Y47*Z47+W47*'01_Cadrage'!$H$24</f>
+        <f>Y47*Z47+W47*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -12001,7 +12068,7 @@
         <v/>
       </c>
       <c r="AA48" s="13">
-        <f>Y48*Z48+W48*'01_Cadrage'!$H$24</f>
+        <f>Y48*Z48+W48*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -12111,7 +12178,7 @@
         <v/>
       </c>
       <c r="AA49" s="13">
-        <f>Y49*Z49+W49*'01_Cadrage'!$H$24</f>
+        <f>Y49*Z49+W49*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -12221,7 +12288,7 @@
         <v/>
       </c>
       <c r="AA50" s="13">
-        <f>Y50*Z50+W50*'01_Cadrage'!$H$24</f>
+        <f>Y50*Z50+W50*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -12331,7 +12398,7 @@
         <v/>
       </c>
       <c r="AA51" s="13">
-        <f>Y51*Z51+W51*'01_Cadrage'!$H$24</f>
+        <f>Y51*Z51+W51*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -12441,7 +12508,7 @@
         <v/>
       </c>
       <c r="AA52" s="13">
-        <f>Y52*Z52+W52*'01_Cadrage'!$H$24</f>
+        <f>Y52*Z52+W52*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -12551,7 +12618,7 @@
         <v/>
       </c>
       <c r="AA53" s="13">
-        <f>Y53*Z53+W53*'01_Cadrage'!$H$24</f>
+        <f>Y53*Z53+W53*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -12661,7 +12728,7 @@
         <v/>
       </c>
       <c r="AA54" s="13">
-        <f>Y54*Z54+W54*'01_Cadrage'!$H$24</f>
+        <f>Y54*Z54+W54*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -12771,7 +12838,7 @@
         <v/>
       </c>
       <c r="AA55" s="13">
-        <f>Y55*Z55+W55*'01_Cadrage'!$H$24</f>
+        <f>Y55*Z55+W55*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -12881,7 +12948,7 @@
         <v/>
       </c>
       <c r="AA56" s="13">
-        <f>Y56*Z56+W56*'01_Cadrage'!$H$24</f>
+        <f>Y56*Z56+W56*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -12991,7 +13058,7 @@
         <v/>
       </c>
       <c r="AA57" s="13">
-        <f>Y57*Z57+W57*'01_Cadrage'!$H$24</f>
+        <f>Y57*Z57+W57*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -13101,7 +13168,7 @@
         <v/>
       </c>
       <c r="AA58" s="13">
-        <f>Y58*Z58+W58*'01_Cadrage'!$H$24</f>
+        <f>Y58*Z58+W58*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -13211,7 +13278,7 @@
         <v/>
       </c>
       <c r="AA59" s="13">
-        <f>Y59*Z59+W59*'01_Cadrage'!$H$24</f>
+        <f>Y59*Z59+W59*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -13321,7 +13388,7 @@
         <v/>
       </c>
       <c r="AA60" s="13">
-        <f>Y60*Z60+W60*'01_Cadrage'!$H$24</f>
+        <f>Y60*Z60+W60*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -13431,7 +13498,7 @@
         <v/>
       </c>
       <c r="AA61" s="13">
-        <f>Y61*Z61+W61*'01_Cadrage'!$H$24</f>
+        <f>Y61*Z61+W61*'01_Cadrage'!$H$26</f>
         <v/>
       </c>
     </row>
@@ -56252,7 +56319,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>COMPTE DE RÉSULTAT (SIG) — réalisé N-2 · réalisé N-1 · atterrissage N</t>
+          <t>COMPTE DE RÉSULTAT (SIG) — réalisé N-2 · N-1 · atterrissage N · BUDGET N+1 (piloté par le cadrage)</t>
         </is>
       </c>
     </row>
@@ -56284,12 +56351,12 @@
       </c>
       <c r="G3" s="10" t="inlineStr">
         <is>
-          <t>Var N-1→N €</t>
+          <t>🟢 Budget N+1</t>
         </is>
       </c>
       <c r="H3" s="10" t="inlineStr">
         <is>
-          <t>Var %</t>
+          <t>Var Bud/Att %</t>
         </is>
       </c>
     </row>
@@ -56329,12 +56396,12 @@
         <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"7062",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G5" s="15">
-        <f>F5-E5</f>
+      <c r="G5" s="53">
+        <f>F5*('04_Moteur'!$AA$62/21936350)</f>
         <v/>
       </c>
       <c r="H5" s="16">
-        <f>IFERROR((F5-E5)/E5,0)</f>
+        <f>IFERROR(G5/F5-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56361,12 +56428,12 @@
         <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"706",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G6" s="15">
-        <f>F6-E6</f>
+      <c r="G6" s="53">
+        <f>F6*('04_Moteur'!$AA$62/21936350)</f>
         <v/>
       </c>
       <c r="H6" s="16">
-        <f>IFERROR((F6-E6)/E6,0)</f>
+        <f>IFERROR(G6/F6-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56393,17 +56460,17 @@
         <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"708",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G7" s="15">
-        <f>F7-E7</f>
+      <c r="G7" s="53">
+        <f>F7*('04_Moteur'!$AA$62/21936350)</f>
         <v/>
       </c>
       <c r="H7" s="16">
-        <f>IFERROR((F7-E7)/E7,0)</f>
+        <f>IFERROR(G7/F7-1,0)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="53" t="inlineStr">
+      <c r="B8" s="54" t="inlineStr">
         <is>
           <t> </t>
         </is>
@@ -56425,12 +56492,12 @@
         <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$H$4:$H$675,"Produit",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G8" s="46">
-        <f>F8-E8</f>
-        <v/>
-      </c>
-      <c r="H8" s="54">
-        <f>IFERROR((F8-E8)/E8,0)</f>
+      <c r="G8" s="55">
+        <f>G5+G6+G7</f>
+        <v/>
+      </c>
+      <c r="H8" s="56">
+        <f>IFERROR(G8/F8-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56470,12 +56537,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"621",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G10" s="15">
-        <f>F10-E10</f>
+      <c r="G10" s="53">
+        <f>F10*('04_Moteur'!$AA$62/21936350)</f>
         <v/>
       </c>
       <c r="H10" s="16">
-        <f>IFERROR((F10-E10)/E10,0)</f>
+        <f>IFERROR(G10/F10-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56502,12 +56569,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"604",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G11" s="15">
-        <f>F11-E11</f>
+      <c r="G11" s="53">
+        <f>F11*('04_Moteur'!$AA$62/21936350)</f>
         <v/>
       </c>
       <c r="H11" s="16">
-        <f>IFERROR((F11-E11)/E11,0)</f>
+        <f>IFERROR(G11/F11-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56534,12 +56601,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"6063",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G12" s="15">
-        <f>F12-E12</f>
+      <c r="G12" s="53">
+        <f>F12*('04_Moteur'!$AA$62/21936350)</f>
         <v/>
       </c>
       <c r="H12" s="16">
-        <f>IFERROR((F12-E12)/E12,0)</f>
+        <f>IFERROR(G12/F12-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56566,17 +56633,17 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"6231",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G13" s="15">
-        <f>F13-E13</f>
+      <c r="G13" s="53">
+        <f>F13*('04_Moteur'!$AA$62/21936350)</f>
         <v/>
       </c>
       <c r="H13" s="16">
-        <f>IFERROR((F13-E13)/E13,0)</f>
+        <f>IFERROR(G13/F13-1,0)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="53" t="inlineStr">
+      <c r="B14" s="54" t="inlineStr">
         <is>
           <t> </t>
         </is>
@@ -56598,12 +56665,12 @@
         <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$H$4:$H$675,"Produit",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$I$4:$I$675,"Coûts directs",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G14" s="46">
-        <f>F14-E14</f>
-        <v/>
-      </c>
-      <c r="H14" s="54">
-        <f>IFERROR((F14-E14)/E14,0)</f>
+      <c r="G14" s="55">
+        <f>G5+G6+G7+G10+G11+G12+G13</f>
+        <v/>
+      </c>
+      <c r="H14" s="56">
+        <f>IFERROR(G14/F14-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56643,12 +56710,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"6411",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G16" s="15">
-        <f>F16-E16</f>
+      <c r="G16" s="53">
+        <f>F16*(('04_Moteur'!$Y$62/2952)*(1+'01_Cadrage'!$H$20))</f>
         <v/>
       </c>
       <c r="H16" s="16">
-        <f>IFERROR((F16-E16)/E16,0)</f>
+        <f>IFERROR(G16/F16-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56675,12 +56742,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"6413",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G17" s="15">
-        <f>F17-E17</f>
+      <c r="G17" s="53">
+        <f>F17*(('04_Moteur'!$Y$62/2952)*(1+'01_Cadrage'!$H$20))</f>
         <v/>
       </c>
       <c r="H17" s="16">
-        <f>IFERROR((F17-E17)/E17,0)</f>
+        <f>IFERROR(G17/F17-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56707,12 +56774,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"6414",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G18" s="15">
-        <f>F18-E18</f>
+      <c r="G18" s="53">
+        <f>F18*(('04_Moteur'!$Y$62/2952)*(1+'01_Cadrage'!$H$20))</f>
         <v/>
       </c>
       <c r="H18" s="16">
-        <f>IFERROR((F18-E18)/E18,0)</f>
+        <f>IFERROR(G18/F18-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56739,12 +56806,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"645",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G19" s="15">
-        <f>F19-E19</f>
+      <c r="G19" s="53">
+        <f>F19*(('04_Moteur'!$Y$62/2952)*(1+'01_Cadrage'!$H$20))</f>
         <v/>
       </c>
       <c r="H19" s="16">
-        <f>IFERROR((F19-E19)/E19,0)</f>
+        <f>IFERROR(G19/F19-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56784,12 +56851,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"613",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G21" s="15">
-        <f>F21-E21</f>
+      <c r="G21" s="53">
+        <f>F21*(1+'01_Cadrage'!$H$19)</f>
         <v/>
       </c>
       <c r="H21" s="16">
-        <f>IFERROR((F21-E21)/E21,0)</f>
+        <f>IFERROR(G21/F21-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56816,12 +56883,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"615",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G22" s="15">
-        <f>F22-E22</f>
+      <c r="G22" s="53">
+        <f>F22*(1+'01_Cadrage'!$H$19)</f>
         <v/>
       </c>
       <c r="H22" s="16">
-        <f>IFERROR((F22-E22)/E22,0)</f>
+        <f>IFERROR(G22/F22-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56848,12 +56915,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"616",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G23" s="15">
-        <f>F23-E23</f>
+      <c r="G23" s="53">
+        <f>F23*(1+'01_Cadrage'!$H$19)</f>
         <v/>
       </c>
       <c r="H23" s="16">
-        <f>IFERROR((F23-E23)/E23,0)</f>
+        <f>IFERROR(G23/F23-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56880,12 +56947,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"6226",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G24" s="15">
-        <f>F24-E24</f>
+      <c r="G24" s="53">
+        <f>F24*(1+'01_Cadrage'!$H$19)</f>
         <v/>
       </c>
       <c r="H24" s="16">
-        <f>IFERROR((F24-E24)/E24,0)</f>
+        <f>IFERROR(G24/F24-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56912,12 +56979,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"6236",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G25" s="15">
-        <f>F25-E25</f>
+      <c r="G25" s="53">
+        <f>F25*(1+'01_Cadrage'!$H$19)</f>
         <v/>
       </c>
       <c r="H25" s="16">
-        <f>IFERROR((F25-E25)/E25,0)</f>
+        <f>IFERROR(G25/F25-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56944,12 +57011,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"625",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G26" s="15">
-        <f>F26-E26</f>
+      <c r="G26" s="53">
+        <f>F26*(1+'01_Cadrage'!$H$19)</f>
         <v/>
       </c>
       <c r="H26" s="16">
-        <f>IFERROR((F26-E26)/E26,0)</f>
+        <f>IFERROR(G26/F26-1,0)</f>
         <v/>
       </c>
     </row>
@@ -56976,12 +57043,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"626",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G27" s="15">
-        <f>F27-E27</f>
+      <c r="G27" s="53">
+        <f>F27*(1+'01_Cadrage'!$H$19)</f>
         <v/>
       </c>
       <c r="H27" s="16">
-        <f>IFERROR((F27-E27)/E27,0)</f>
+        <f>IFERROR(G27/F27-1,0)</f>
         <v/>
       </c>
     </row>
@@ -57008,12 +57075,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"6281",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G28" s="15">
-        <f>F28-E28</f>
+      <c r="G28" s="53">
+        <f>F28*(1+'01_Cadrage'!$H$19)</f>
         <v/>
       </c>
       <c r="H28" s="16">
-        <f>IFERROR((F28-E28)/E28,0)</f>
+        <f>IFERROR(G28/F28-1,0)</f>
         <v/>
       </c>
     </row>
@@ -57053,12 +57120,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"6331",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G30" s="15">
-        <f>F30-E30</f>
+      <c r="G30" s="53">
+        <f>F30*(1+'01_Cadrage'!$H$19)</f>
         <v/>
       </c>
       <c r="H30" s="16">
-        <f>IFERROR((F30-E30)/E30,0)</f>
+        <f>IFERROR(G30/F30-1,0)</f>
         <v/>
       </c>
     </row>
@@ -57085,12 +57152,12 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"63511",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G31" s="15">
-        <f>F31-E31</f>
+      <c r="G31" s="53">
+        <f>F31*(1+'01_Cadrage'!$H$19)</f>
         <v/>
       </c>
       <c r="H31" s="16">
-        <f>IFERROR((F31-E31)/E31,0)</f>
+        <f>IFERROR(G31/F31-1,0)</f>
         <v/>
       </c>
     </row>
@@ -57117,17 +57184,17 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"6333",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G32" s="15">
-        <f>F32-E32</f>
+      <c r="G32" s="53">
+        <f>F32*(1+'01_Cadrage'!$H$19)</f>
         <v/>
       </c>
       <c r="H32" s="16">
-        <f>IFERROR((F32-E32)/E32,0)</f>
+        <f>IFERROR(G32/F32-1,0)</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="53" t="inlineStr">
+      <c r="B33" s="54" t="inlineStr">
         <is>
           <t> </t>
         </is>
@@ -57149,12 +57216,12 @@
         <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$H$4:$H$675,"Produit",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$H$4:$H$675,"Charge",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")+SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$I$4:$I$675,"Dotations",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G33" s="46">
-        <f>F33-E33</f>
-        <v/>
-      </c>
-      <c r="H33" s="54">
-        <f>IFERROR((F33-E33)/E33,0)</f>
+      <c r="G33" s="55">
+        <f>G5+G6+G7+G10+G11+G12+G13+G16+G17+G18+G19+G21+G22+G23+G24+G25+G26+G27+G28+G30+G31+G32</f>
+        <v/>
+      </c>
+      <c r="H33" s="56">
+        <f>IFERROR(G33/F33-1,0)</f>
         <v/>
       </c>
     </row>
@@ -57194,17 +57261,17 @@
         <f>-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$E$4:$E$675,"6811",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G35" s="15">
-        <f>F35-E35</f>
+      <c r="G35" s="53">
+        <f>F35*(1+'01_Cadrage'!$H$19)</f>
         <v/>
       </c>
       <c r="H35" s="16">
-        <f>IFERROR((F35-E35)/E35,0)</f>
+        <f>IFERROR(G35/F35-1,0)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="53" t="inlineStr">
+      <c r="B36" s="54" t="inlineStr">
         <is>
           <t> </t>
         </is>
@@ -57226,12 +57293,12 @@
         <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$H$4:$H$675,"Produit",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$H$4:$H$675,"Charge",'06_Compta'!$J$4:$J$675,"2025ATT_VDEF")</f>
         <v/>
       </c>
-      <c r="G36" s="46">
-        <f>F36-E36</f>
-        <v/>
-      </c>
-      <c r="H36" s="54">
-        <f>IFERROR((F36-E36)/E36,0)</f>
+      <c r="G36" s="55">
+        <f>G5+G6+G7+G10+G11+G12+G13+G16+G17+G18+G19+G21+G22+G23+G24+G25+G26+G27+G28+G30+G31+G32+G35</f>
+        <v/>
+      </c>
+      <c r="H36" s="56">
+        <f>IFERROR(G36/F36-1,0)</f>
         <v/>
       </c>
     </row>
@@ -57241,16 +57308,20 @@
           <t>Marge EBITDA %</t>
         </is>
       </c>
-      <c r="D37" s="55">
+      <c r="D37" s="57">
         <f>IFERROR(D33/D8,0)</f>
         <v/>
       </c>
-      <c r="E37" s="55">
+      <c r="E37" s="57">
         <f>IFERROR(E33/E8,0)</f>
         <v/>
       </c>
-      <c r="F37" s="55">
+      <c r="F37" s="57">
         <f>IFERROR(F33/F8,0)</f>
+        <v/>
+      </c>
+      <c r="G37" s="57">
+        <f>IFERROR(G33/G8,0)</f>
         <v/>
       </c>
     </row>
@@ -57260,16 +57331,20 @@
           <t>Marge EBIT %</t>
         </is>
       </c>
-      <c r="D38" s="55">
+      <c r="D38" s="57">
         <f>IFERROR(D36/D8,0)</f>
         <v/>
       </c>
-      <c r="E38" s="55">
+      <c r="E38" s="57">
         <f>IFERROR(E36/E8,0)</f>
         <v/>
       </c>
-      <c r="F38" s="55">
+      <c r="F38" s="57">
         <f>IFERROR(F36/F8,0)</f>
+        <v/>
+      </c>
+      <c r="G38" s="57">
+        <f>IFERROR(G36/G8,0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Part organique & rendement différenciés par campus + indicateur d'attractivité
- part organique différenciée (30%→53%) : force de marque ↑ / concurrence ville ↓
- rendement d'acquisition différencié (0,42→0,59) : sophistication marketing +
  marge de marché — mesuré depuis un historique CRM généré en conséquence
- 03_Campagnes : indicateur d'ATTRACTIVITÉ = CAC marginal (CPL ÷ rendement ÷
  conversion) avec échelle de couleur vert→rouge = où l'euro marketing rapporte
  · MBway Bordeaux 890 € (investir) vs Tunon Paris 2 193 € (cher & inefficace)
- tout reste connecté : le moteur consomme le rendement mesuré par campus →
  impact marketing différencié par école
- 0 erreur

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_CA_v3.xlsx
+++ b/eduservices/EDUSERVICES_Modele_CA_v3.xlsx
@@ -6227,17 +6227,17 @@
         <v>2024</v>
       </c>
       <c r="E4" s="24" t="n">
-        <v>717</v>
+        <v>645</v>
       </c>
       <c r="F4" s="24" t="n">
-        <v>1078</v>
+        <v>1158</v>
       </c>
       <c r="G4" s="27">
         <f>E4+F4</f>
         <v/>
       </c>
       <c r="H4" s="12" t="n">
-        <v>52911</v>
+        <v>56438</v>
       </c>
     </row>
     <row r="5">
@@ -6259,17 +6259,17 @@
         <v>2025</v>
       </c>
       <c r="E5" s="24" t="n">
-        <v>753</v>
+        <v>677</v>
       </c>
       <c r="F5" s="24" t="n">
-        <v>1130</v>
+        <v>1210</v>
       </c>
       <c r="G5" s="27">
         <f>E5+F5</f>
         <v/>
       </c>
       <c r="H5" s="12" t="n">
-        <v>58202</v>
+        <v>62082</v>
       </c>
     </row>
     <row r="6">
@@ -6291,17 +6291,17 @@
         <v>2026</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>790</v>
+        <v>711</v>
       </c>
       <c r="F6" s="24" t="n">
-        <v>1186</v>
+        <v>1265</v>
       </c>
       <c r="G6" s="27">
         <f>E6+F6</f>
         <v/>
       </c>
       <c r="H6" s="12" t="n">
-        <v>64022</v>
+        <v>68291</v>
       </c>
     </row>
     <row r="7">
@@ -6323,17 +6323,17 @@
         <v>2024</v>
       </c>
       <c r="E7" s="24" t="n">
-        <v>604</v>
+        <v>650</v>
       </c>
       <c r="F7" s="24" t="n">
-        <v>909</v>
+        <v>863</v>
       </c>
       <c r="G7" s="27">
         <f>E7+F7</f>
         <v/>
       </c>
       <c r="H7" s="12" t="n">
-        <v>36349</v>
+        <v>34532</v>
       </c>
     </row>
     <row r="8">
@@ -6355,17 +6355,17 @@
         <v>2025</v>
       </c>
       <c r="E8" s="24" t="n">
-        <v>635</v>
+        <v>682</v>
       </c>
       <c r="F8" s="24" t="n">
-        <v>953</v>
+        <v>905</v>
       </c>
       <c r="G8" s="27">
         <f>E8+F8</f>
         <v/>
       </c>
       <c r="H8" s="12" t="n">
-        <v>39984</v>
+        <v>37985</v>
       </c>
     </row>
     <row r="9">
@@ -6387,17 +6387,17 @@
         <v>2026</v>
       </c>
       <c r="E9" s="24" t="n">
-        <v>666</v>
+        <v>716</v>
       </c>
       <c r="F9" s="24" t="n">
-        <v>1000</v>
+        <v>950</v>
       </c>
       <c r="G9" s="27">
         <f>E9+F9</f>
         <v/>
       </c>
       <c r="H9" s="12" t="n">
-        <v>43982</v>
+        <v>41783</v>
       </c>
     </row>
     <row r="10">
@@ -6419,17 +6419,17 @@
         <v>2024</v>
       </c>
       <c r="E10" s="24" t="n">
-        <v>550</v>
+        <v>660</v>
       </c>
       <c r="F10" s="24" t="n">
-        <v>827</v>
+        <v>713</v>
       </c>
       <c r="G10" s="27">
         <f>E10+F10</f>
         <v/>
       </c>
       <c r="H10" s="12" t="n">
-        <v>30069</v>
+        <v>26060</v>
       </c>
     </row>
     <row r="11">
@@ -6451,17 +6451,17 @@
         <v>2025</v>
       </c>
       <c r="E11" s="24" t="n">
-        <v>578</v>
+        <v>693</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>867</v>
+        <v>749</v>
       </c>
       <c r="G11" s="27">
         <f>E11+F11</f>
         <v/>
       </c>
       <c r="H11" s="12" t="n">
-        <v>33076</v>
+        <v>28666</v>
       </c>
     </row>
     <row r="12">
@@ -6483,17 +6483,17 @@
         <v>2026</v>
       </c>
       <c r="E12" s="24" t="n">
-        <v>606</v>
+        <v>728</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>910</v>
+        <v>788</v>
       </c>
       <c r="G12" s="27">
         <f>E12+F12</f>
         <v/>
       </c>
       <c r="H12" s="12" t="n">
-        <v>36384</v>
+        <v>31533</v>
       </c>
     </row>
     <row r="13">
@@ -6515,17 +6515,17 @@
         <v>2024</v>
       </c>
       <c r="E13" s="24" t="n">
-        <v>467</v>
+        <v>572</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>701</v>
+        <v>592</v>
       </c>
       <c r="G13" s="27">
         <f>E13+F13</f>
         <v/>
       </c>
       <c r="H13" s="12" t="n">
-        <v>24232</v>
+        <v>20597</v>
       </c>
     </row>
     <row r="14">
@@ -6547,17 +6547,17 @@
         <v>2025</v>
       </c>
       <c r="E14" s="24" t="n">
-        <v>490</v>
+        <v>600</v>
       </c>
       <c r="F14" s="24" t="n">
-        <v>736</v>
+        <v>623</v>
       </c>
       <c r="G14" s="27">
         <f>E14+F14</f>
         <v/>
       </c>
       <c r="H14" s="12" t="n">
-        <v>26655</v>
+        <v>22657</v>
       </c>
     </row>
     <row r="15">
@@ -6579,17 +6579,17 @@
         <v>2026</v>
       </c>
       <c r="E15" s="24" t="n">
-        <v>514</v>
+        <v>630</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>772</v>
+        <v>656</v>
       </c>
       <c r="G15" s="27">
         <f>E15+F15</f>
         <v/>
       </c>
       <c r="H15" s="12" t="n">
-        <v>29321</v>
+        <v>24923</v>
       </c>
     </row>
     <row r="16">
@@ -6611,17 +6611,17 @@
         <v>2024</v>
       </c>
       <c r="E16" s="24" t="n">
-        <v>659</v>
+        <v>626</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>991</v>
+        <v>1035</v>
       </c>
       <c r="G16" s="27">
         <f>E16+F16</f>
         <v/>
       </c>
       <c r="H16" s="12" t="n">
-        <v>48627</v>
+        <v>50248</v>
       </c>
     </row>
     <row r="17">
@@ -6643,17 +6643,17 @@
         <v>2025</v>
       </c>
       <c r="E17" s="24" t="n">
-        <v>692</v>
+        <v>657</v>
       </c>
       <c r="F17" s="24" t="n">
-        <v>1039</v>
+        <v>1080</v>
       </c>
       <c r="G17" s="27">
         <f>E17+F17</f>
         <v/>
       </c>
       <c r="H17" s="12" t="n">
-        <v>53489</v>
+        <v>55272</v>
       </c>
     </row>
     <row r="18">
@@ -6675,17 +6675,17 @@
         <v>2026</v>
       </c>
       <c r="E18" s="24" t="n">
-        <v>726</v>
+        <v>690</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>1090</v>
+        <v>1126</v>
       </c>
       <c r="G18" s="27">
         <f>E18+F18</f>
         <v/>
       </c>
       <c r="H18" s="12" t="n">
-        <v>58838</v>
+        <v>60800</v>
       </c>
     </row>
     <row r="19">
@@ -6707,17 +6707,17 @@
         <v>2024</v>
       </c>
       <c r="E19" s="24" t="n">
-        <v>458</v>
+        <v>572</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>688</v>
+        <v>571</v>
       </c>
       <c r="G19" s="27">
         <f>E19+F19</f>
         <v/>
       </c>
       <c r="H19" s="12" t="n">
-        <v>25012</v>
+        <v>20843</v>
       </c>
     </row>
     <row r="20">
@@ -6739,17 +6739,17 @@
         <v>2025</v>
       </c>
       <c r="E20" s="24" t="n">
-        <v>480</v>
+        <v>600</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>721</v>
+        <v>600</v>
       </c>
       <c r="G20" s="27">
         <f>E20+F20</f>
         <v/>
       </c>
       <c r="H20" s="12" t="n">
-        <v>27513</v>
+        <v>22927</v>
       </c>
     </row>
     <row r="21">
@@ -6771,17 +6771,17 @@
         <v>2026</v>
       </c>
       <c r="E21" s="24" t="n">
-        <v>504</v>
+        <v>630</v>
       </c>
       <c r="F21" s="24" t="n">
-        <v>757</v>
+        <v>630</v>
       </c>
       <c r="G21" s="27">
         <f>E21+F21</f>
         <v/>
       </c>
       <c r="H21" s="12" t="n">
-        <v>30264</v>
+        <v>25220</v>
       </c>
     </row>
     <row r="22">
@@ -6803,17 +6803,17 @@
         <v>2024</v>
       </c>
       <c r="E22" s="24" t="n">
-        <v>430</v>
+        <v>549</v>
       </c>
       <c r="F22" s="24" t="n">
-        <v>647</v>
+        <v>526</v>
       </c>
       <c r="G22" s="27">
         <f>E22+F22</f>
         <v/>
       </c>
       <c r="H22" s="12" t="n">
-        <v>22348</v>
+        <v>18251</v>
       </c>
     </row>
     <row r="23">
@@ -6835,17 +6835,17 @@
         <v>2025</v>
       </c>
       <c r="E23" s="24" t="n">
-        <v>452</v>
+        <v>576</v>
       </c>
       <c r="F23" s="24" t="n">
-        <v>678</v>
+        <v>553</v>
       </c>
       <c r="G23" s="27">
         <f>E23+F23</f>
         <v/>
       </c>
       <c r="H23" s="12" t="n">
-        <v>24583</v>
+        <v>20076</v>
       </c>
     </row>
     <row r="24">
@@ -6867,17 +6867,17 @@
         <v>2026</v>
       </c>
       <c r="E24" s="24" t="n">
-        <v>474</v>
+        <v>605</v>
       </c>
       <c r="F24" s="24" t="n">
-        <v>712</v>
+        <v>581</v>
       </c>
       <c r="G24" s="27">
         <f>E24+F24</f>
         <v/>
       </c>
       <c r="H24" s="12" t="n">
-        <v>27041</v>
+        <v>22083</v>
       </c>
     </row>
     <row r="25">
@@ -6899,17 +6899,17 @@
         <v>2024</v>
       </c>
       <c r="E25" s="24" t="n">
-        <v>308</v>
+        <v>278</v>
       </c>
       <c r="F25" s="24" t="n">
-        <v>464</v>
+        <v>489</v>
       </c>
       <c r="G25" s="27">
         <f>E25+F25</f>
         <v/>
       </c>
       <c r="H25" s="12" t="n">
-        <v>16860</v>
+        <v>17983</v>
       </c>
     </row>
     <row r="26">
@@ -6931,17 +6931,17 @@
         <v>2025</v>
       </c>
       <c r="E26" s="24" t="n">
-        <v>324</v>
+        <v>291</v>
       </c>
       <c r="F26" s="24" t="n">
-        <v>486</v>
+        <v>516</v>
       </c>
       <c r="G26" s="27">
         <f>E26+F26</f>
         <v/>
       </c>
       <c r="H26" s="12" t="n">
-        <v>18545</v>
+        <v>19782</v>
       </c>
     </row>
     <row r="27">
@@ -6963,17 +6963,17 @@
         <v>2026</v>
       </c>
       <c r="E27" s="24" t="n">
-        <v>340</v>
+        <v>306</v>
       </c>
       <c r="F27" s="24" t="n">
-        <v>510</v>
+        <v>544</v>
       </c>
       <c r="G27" s="27">
         <f>E27+F27</f>
         <v/>
       </c>
       <c r="H27" s="12" t="n">
-        <v>20400</v>
+        <v>21760</v>
       </c>
     </row>
     <row r="28">
@@ -6995,7 +6995,7 @@
         <v>2024</v>
       </c>
       <c r="E28" s="24" t="n">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="F28" s="24" t="n">
         <v>371</v>
@@ -7005,7 +7005,7 @@
         <v/>
       </c>
       <c r="H28" s="12" t="n">
-        <v>12139</v>
+        <v>12341</v>
       </c>
     </row>
     <row r="29">
@@ -7027,17 +7027,17 @@
         <v>2025</v>
       </c>
       <c r="E29" s="24" t="n">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="G29" s="27">
         <f>E29+F29</f>
         <v/>
       </c>
       <c r="H29" s="12" t="n">
-        <v>13353</v>
+        <v>13575</v>
       </c>
     </row>
     <row r="30">
@@ -7059,17 +7059,17 @@
         <v>2026</v>
       </c>
       <c r="E30" s="24" t="n">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="F30" s="24" t="n">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="G30" s="27">
         <f>E30+F30</f>
         <v/>
       </c>
       <c r="H30" s="12" t="n">
-        <v>14688</v>
+        <v>14933</v>
       </c>
     </row>
     <row r="31">
@@ -7091,17 +7091,17 @@
         <v>2024</v>
       </c>
       <c r="E31" s="24" t="n">
-        <v>247</v>
+        <v>234</v>
       </c>
       <c r="F31" s="24" t="n">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="G31" s="27">
         <f>E31+F31</f>
         <v/>
       </c>
       <c r="H31" s="12" t="n">
-        <v>12139</v>
+        <v>12543</v>
       </c>
     </row>
     <row r="32">
@@ -7123,17 +7123,17 @@
         <v>2025</v>
       </c>
       <c r="E32" s="24" t="n">
-        <v>259</v>
+        <v>246</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>389</v>
+        <v>399</v>
       </c>
       <c r="G32" s="27">
         <f>E32+F32</f>
         <v/>
       </c>
       <c r="H32" s="12" t="n">
-        <v>13353</v>
+        <v>13798</v>
       </c>
     </row>
     <row r="33">
@@ -7155,17 +7155,17 @@
         <v>2026</v>
       </c>
       <c r="E33" s="24" t="n">
-        <v>272</v>
+        <v>258</v>
       </c>
       <c r="F33" s="24" t="n">
-        <v>408</v>
+        <v>422</v>
       </c>
       <c r="G33" s="27">
         <f>E33+F33</f>
         <v/>
       </c>
       <c r="H33" s="12" t="n">
-        <v>14688</v>
+        <v>15178</v>
       </c>
     </row>
     <row r="34">
@@ -7187,17 +7187,17 @@
         <v>2024</v>
       </c>
       <c r="E34" s="24" t="n">
-        <v>570</v>
+        <v>669</v>
       </c>
       <c r="F34" s="24" t="n">
-        <v>856</v>
+        <v>765</v>
       </c>
       <c r="G34" s="27">
         <f>E34+F34</f>
         <v/>
       </c>
       <c r="H34" s="12" t="n">
-        <v>34255</v>
+        <v>30258</v>
       </c>
     </row>
     <row r="35">
@@ -7219,17 +7219,17 @@
         <v>2025</v>
       </c>
       <c r="E35" s="24" t="n">
-        <v>598</v>
+        <v>703</v>
       </c>
       <c r="F35" s="24" t="n">
-        <v>898</v>
+        <v>798</v>
       </c>
       <c r="G35" s="27">
         <f>E35+F35</f>
         <v/>
       </c>
       <c r="H35" s="12" t="n">
-        <v>37680</v>
+        <v>33284</v>
       </c>
     </row>
     <row r="36">
@@ -7251,17 +7251,17 @@
         <v>2026</v>
       </c>
       <c r="E36" s="24" t="n">
-        <v>628</v>
+        <v>738</v>
       </c>
       <c r="F36" s="24" t="n">
-        <v>942</v>
+        <v>832</v>
       </c>
       <c r="G36" s="27">
         <f>E36+F36</f>
         <v/>
       </c>
       <c r="H36" s="12" t="n">
-        <v>41448</v>
+        <v>36612</v>
       </c>
     </row>
     <row r="37">
@@ -7283,17 +7283,17 @@
         <v>2024</v>
       </c>
       <c r="E37" s="24" t="n">
-        <v>446</v>
+        <v>591</v>
       </c>
       <c r="F37" s="24" t="n">
-        <v>671</v>
+        <v>528</v>
       </c>
       <c r="G37" s="27">
         <f>E37+F37</f>
         <v/>
       </c>
       <c r="H37" s="12" t="n">
-        <v>23177</v>
+        <v>18155</v>
       </c>
     </row>
     <row r="38">
@@ -7315,17 +7315,17 @@
         <v>2025</v>
       </c>
       <c r="E38" s="24" t="n">
-        <v>469</v>
+        <v>621</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>704</v>
+        <v>552</v>
       </c>
       <c r="G38" s="27">
         <f>E38+F38</f>
         <v/>
       </c>
       <c r="H38" s="12" t="n">
-        <v>25495</v>
+        <v>19971</v>
       </c>
     </row>
     <row r="39">
@@ -7347,17 +7347,17 @@
         <v>2026</v>
       </c>
       <c r="E39" s="24" t="n">
-        <v>492</v>
+        <v>652</v>
       </c>
       <c r="F39" s="24" t="n">
-        <v>738</v>
+        <v>578</v>
       </c>
       <c r="G39" s="27">
         <f>E39+F39</f>
         <v/>
       </c>
       <c r="H39" s="12" t="n">
-        <v>28044</v>
+        <v>21968</v>
       </c>
     </row>
     <row r="40">
@@ -7379,17 +7379,17 @@
         <v>2024</v>
       </c>
       <c r="E40" s="24" t="n">
-        <v>290</v>
+        <v>218</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>436</v>
+        <v>517</v>
       </c>
       <c r="G40" s="27">
         <f>E40+F40</f>
         <v/>
       </c>
       <c r="H40" s="12" t="n">
-        <v>21421</v>
+        <v>24992</v>
       </c>
     </row>
     <row r="41">
@@ -7411,17 +7411,17 @@
         <v>2025</v>
       </c>
       <c r="E41" s="24" t="n">
-        <v>305</v>
+        <v>229</v>
       </c>
       <c r="F41" s="24" t="n">
-        <v>458</v>
+        <v>538</v>
       </c>
       <c r="G41" s="27">
         <f>E41+F41</f>
         <v/>
       </c>
       <c r="H41" s="12" t="n">
-        <v>23564</v>
+        <v>27491</v>
       </c>
     </row>
     <row r="42">
@@ -7443,17 +7443,17 @@
         <v>2026</v>
       </c>
       <c r="E42" s="24" t="n">
-        <v>320</v>
+        <v>240</v>
       </c>
       <c r="F42" s="24" t="n">
-        <v>480</v>
+        <v>560</v>
       </c>
       <c r="G42" s="27">
         <f>E42+F42</f>
         <v/>
       </c>
       <c r="H42" s="12" t="n">
-        <v>25920</v>
+        <v>30240</v>
       </c>
     </row>
     <row r="43">
@@ -7475,17 +7475,17 @@
         <v>2024</v>
       </c>
       <c r="E43" s="24" t="n">
-        <v>247</v>
+        <v>228</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>371</v>
+        <v>392</v>
       </c>
       <c r="G43" s="27">
         <f>E43+F43</f>
         <v/>
       </c>
       <c r="H43" s="12" t="n">
-        <v>14836</v>
+        <v>15578</v>
       </c>
     </row>
     <row r="44">
@@ -7507,17 +7507,17 @@
         <v>2025</v>
       </c>
       <c r="E44" s="24" t="n">
-        <v>259</v>
+        <v>240</v>
       </c>
       <c r="F44" s="24" t="n">
-        <v>389</v>
+        <v>410</v>
       </c>
       <c r="G44" s="27">
         <f>E44+F44</f>
         <v/>
       </c>
       <c r="H44" s="12" t="n">
-        <v>16320</v>
+        <v>17136</v>
       </c>
     </row>
     <row r="45">
@@ -7539,17 +7539,17 @@
         <v>2026</v>
       </c>
       <c r="E45" s="24" t="n">
-        <v>272</v>
+        <v>252</v>
       </c>
       <c r="F45" s="24" t="n">
-        <v>408</v>
+        <v>428</v>
       </c>
       <c r="G45" s="27">
         <f>E45+F45</f>
         <v/>
       </c>
       <c r="H45" s="12" t="n">
-        <v>17952</v>
+        <v>18850</v>
       </c>
     </row>
   </sheetData>
@@ -7567,7 +7567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -7584,6 +7584,8 @@
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -7671,6 +7673,16 @@
           <t>CPL effectif</t>
         </is>
       </c>
+      <c r="O3" s="10" t="inlineStr">
+        <is>
+          <t>Conv. lead→inscrit</t>
+        </is>
+      </c>
+      <c r="P3" s="10" t="inlineStr">
+        <is>
+          <t>CAC marginal /inscrit</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
@@ -7731,6 +7743,14 @@
         <f>IFERROR(K5/L5,0)</f>
         <v/>
       </c>
+      <c r="O5" s="42">
+        <f>IFERROR(SUMIFS('02_Base'!$K$4:$K$61,'02_Base'!$A$4:$A$61,A5,'02_Base'!$B$4:$B$61,B5,'02_Base'!$G$4:$G$61,1)/SUMIFS('02_Base'!$H$4:$H$61,'02_Base'!$A$4:$A$61,A5,'02_Base'!$B$4:$B$61,B5,'02_Base'!$G$4:$G$61,1),0)</f>
+        <v/>
+      </c>
+      <c r="P5" s="13">
+        <f>IFERROR(I5/(J5*O5),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="inlineStr">
@@ -7791,6 +7811,14 @@
         <f>IFERROR(K6/L6,0)</f>
         <v/>
       </c>
+      <c r="O6" s="42">
+        <f>IFERROR(SUMIFS('02_Base'!$K$4:$K$61,'02_Base'!$A$4:$A$61,A6,'02_Base'!$B$4:$B$61,B6,'02_Base'!$G$4:$G$61,1)/SUMIFS('02_Base'!$H$4:$H$61,'02_Base'!$A$4:$A$61,A6,'02_Base'!$B$4:$B$61,B6,'02_Base'!$G$4:$G$61,1),0)</f>
+        <v/>
+      </c>
+      <c r="P6" s="13">
+        <f>IFERROR(I6/(J6*O6),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
@@ -7851,6 +7879,14 @@
         <f>IFERROR(K7/L7,0)</f>
         <v/>
       </c>
+      <c r="O7" s="42">
+        <f>IFERROR(SUMIFS('02_Base'!$K$4:$K$61,'02_Base'!$A$4:$A$61,A7,'02_Base'!$B$4:$B$61,B7,'02_Base'!$G$4:$G$61,1)/SUMIFS('02_Base'!$H$4:$H$61,'02_Base'!$A$4:$A$61,A7,'02_Base'!$B$4:$B$61,B7,'02_Base'!$G$4:$G$61,1),0)</f>
+        <v/>
+      </c>
+      <c r="P7" s="13">
+        <f>IFERROR(I7/(J7*O7),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="17" t="inlineStr">
@@ -7911,6 +7947,14 @@
         <f>IFERROR(K8/L8,0)</f>
         <v/>
       </c>
+      <c r="O8" s="42">
+        <f>IFERROR(SUMIFS('02_Base'!$K$4:$K$61,'02_Base'!$A$4:$A$61,A8,'02_Base'!$B$4:$B$61,B8,'02_Base'!$G$4:$G$61,1)/SUMIFS('02_Base'!$H$4:$H$61,'02_Base'!$A$4:$A$61,A8,'02_Base'!$B$4:$B$61,B8,'02_Base'!$G$4:$G$61,1),0)</f>
+        <v/>
+      </c>
+      <c r="P8" s="13">
+        <f>IFERROR(I8/(J8*O8),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="17" t="inlineStr">
@@ -7971,6 +8015,14 @@
         <f>IFERROR(K9/L9,0)</f>
         <v/>
       </c>
+      <c r="O9" s="42">
+        <f>IFERROR(SUMIFS('02_Base'!$K$4:$K$61,'02_Base'!$A$4:$A$61,A9,'02_Base'!$B$4:$B$61,B9,'02_Base'!$G$4:$G$61,1)/SUMIFS('02_Base'!$H$4:$H$61,'02_Base'!$A$4:$A$61,A9,'02_Base'!$B$4:$B$61,B9,'02_Base'!$G$4:$G$61,1),0)</f>
+        <v/>
+      </c>
+      <c r="P9" s="13">
+        <f>IFERROR(I9/(J9*O9),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="inlineStr">
@@ -8031,6 +8083,14 @@
         <f>IFERROR(K10/L10,0)</f>
         <v/>
       </c>
+      <c r="O10" s="42">
+        <f>IFERROR(SUMIFS('02_Base'!$K$4:$K$61,'02_Base'!$A$4:$A$61,A10,'02_Base'!$B$4:$B$61,B10,'02_Base'!$G$4:$G$61,1)/SUMIFS('02_Base'!$H$4:$H$61,'02_Base'!$A$4:$A$61,A10,'02_Base'!$B$4:$B$61,B10,'02_Base'!$G$4:$G$61,1),0)</f>
+        <v/>
+      </c>
+      <c r="P10" s="13">
+        <f>IFERROR(I10/(J10*O10),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
@@ -8091,6 +8151,14 @@
         <f>IFERROR(K11/L11,0)</f>
         <v/>
       </c>
+      <c r="O11" s="42">
+        <f>IFERROR(SUMIFS('02_Base'!$K$4:$K$61,'02_Base'!$A$4:$A$61,A11,'02_Base'!$B$4:$B$61,B11,'02_Base'!$G$4:$G$61,1)/SUMIFS('02_Base'!$H$4:$H$61,'02_Base'!$A$4:$A$61,A11,'02_Base'!$B$4:$B$61,B11,'02_Base'!$G$4:$G$61,1),0)</f>
+        <v/>
+      </c>
+      <c r="P11" s="13">
+        <f>IFERROR(I11/(J11*O11),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="17" t="inlineStr">
@@ -8151,6 +8219,14 @@
         <f>IFERROR(K12/L12,0)</f>
         <v/>
       </c>
+      <c r="O12" s="42">
+        <f>IFERROR(SUMIFS('02_Base'!$K$4:$K$61,'02_Base'!$A$4:$A$61,A12,'02_Base'!$B$4:$B$61,B12,'02_Base'!$G$4:$G$61,1)/SUMIFS('02_Base'!$H$4:$H$61,'02_Base'!$A$4:$A$61,A12,'02_Base'!$B$4:$B$61,B12,'02_Base'!$G$4:$G$61,1),0)</f>
+        <v/>
+      </c>
+      <c r="P12" s="13">
+        <f>IFERROR(I12/(J12*O12),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
@@ -8211,6 +8287,14 @@
         <f>IFERROR(K13/L13,0)</f>
         <v/>
       </c>
+      <c r="O13" s="42">
+        <f>IFERROR(SUMIFS('02_Base'!$K$4:$K$61,'02_Base'!$A$4:$A$61,A13,'02_Base'!$B$4:$B$61,B13,'02_Base'!$G$4:$G$61,1)/SUMIFS('02_Base'!$H$4:$H$61,'02_Base'!$A$4:$A$61,A13,'02_Base'!$B$4:$B$61,B13,'02_Base'!$G$4:$G$61,1),0)</f>
+        <v/>
+      </c>
+      <c r="P13" s="13">
+        <f>IFERROR(I13/(J13*O13),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="17" t="inlineStr">
@@ -8271,6 +8355,14 @@
         <f>IFERROR(K14/L14,0)</f>
         <v/>
       </c>
+      <c r="O14" s="42">
+        <f>IFERROR(SUMIFS('02_Base'!$K$4:$K$61,'02_Base'!$A$4:$A$61,A14,'02_Base'!$B$4:$B$61,B14,'02_Base'!$G$4:$G$61,1)/SUMIFS('02_Base'!$H$4:$H$61,'02_Base'!$A$4:$A$61,A14,'02_Base'!$B$4:$B$61,B14,'02_Base'!$G$4:$G$61,1),0)</f>
+        <v/>
+      </c>
+      <c r="P14" s="13">
+        <f>IFERROR(I14/(J14*O14),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
@@ -8331,6 +8423,14 @@
         <f>IFERROR(K15/L15,0)</f>
         <v/>
       </c>
+      <c r="O15" s="42">
+        <f>IFERROR(SUMIFS('02_Base'!$K$4:$K$61,'02_Base'!$A$4:$A$61,A15,'02_Base'!$B$4:$B$61,B15,'02_Base'!$G$4:$G$61,1)/SUMIFS('02_Base'!$H$4:$H$61,'02_Base'!$A$4:$A$61,A15,'02_Base'!$B$4:$B$61,B15,'02_Base'!$G$4:$G$61,1),0)</f>
+        <v/>
+      </c>
+      <c r="P15" s="13">
+        <f>IFERROR(I15/(J15*O15),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="17" t="inlineStr">
@@ -8391,6 +8491,14 @@
         <f>IFERROR(K16/L16,0)</f>
         <v/>
       </c>
+      <c r="O16" s="42">
+        <f>IFERROR(SUMIFS('02_Base'!$K$4:$K$61,'02_Base'!$A$4:$A$61,A16,'02_Base'!$B$4:$B$61,B16,'02_Base'!$G$4:$G$61,1)/SUMIFS('02_Base'!$H$4:$H$61,'02_Base'!$A$4:$A$61,A16,'02_Base'!$B$4:$B$61,B16,'02_Base'!$G$4:$G$61,1),0)</f>
+        <v/>
+      </c>
+      <c r="P16" s="13">
+        <f>IFERROR(I16/(J16*O16),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
@@ -8451,6 +8559,14 @@
         <f>IFERROR(K17/L17,0)</f>
         <v/>
       </c>
+      <c r="O17" s="42">
+        <f>IFERROR(SUMIFS('02_Base'!$K$4:$K$61,'02_Base'!$A$4:$A$61,A17,'02_Base'!$B$4:$B$61,B17,'02_Base'!$G$4:$G$61,1)/SUMIFS('02_Base'!$H$4:$H$61,'02_Base'!$A$4:$A$61,A17,'02_Base'!$B$4:$B$61,B17,'02_Base'!$G$4:$G$61,1),0)</f>
+        <v/>
+      </c>
+      <c r="P17" s="13">
+        <f>IFERROR(I17/(J17*O17),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
@@ -8511,12 +8627,40 @@
         <f>IFERROR(K18/L18,0)</f>
         <v/>
       </c>
+      <c r="O18" s="42">
+        <f>IFERROR(SUMIFS('02_Base'!$K$4:$K$61,'02_Base'!$A$4:$A$61,A18,'02_Base'!$B$4:$B$61,B18,'02_Base'!$G$4:$G$61,1)/SUMIFS('02_Base'!$H$4:$H$61,'02_Base'!$A$4:$A$61,A18,'02_Base'!$B$4:$B$61,B18,'02_Base'!$G$4:$G$61,1),0)</f>
+        <v/>
+      </c>
+      <c r="P18" s="13">
+        <f>IFERROR(I18/(J18*O18),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>Indicateur d'attractivité : CAC marginal = coût marketing du prochain inscrit. Vert = investir ici (l'euro rapporte) · Rouge = marché cher/saturé.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A1:N1"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A20:P20"/>
+    <mergeCell ref="A2:P2"/>
   </mergeCells>
+  <conditionalFormatting sqref="P5:P18">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Reporting : KPIs d'impact live + ponts de variance CA & EBITDA
- 09_Reporting : 8 tuiles KPI qui se recalculent en direct (CA, EBITDA, marge,
  effectif, écart cible, reste à trouver, CPL moyen, CAC/inscrit)
- pont CA (tie-out exact) : Référence + effet volume + effet prix&mix = construit
- pont EBITDA (tie-out) : Référence + effet CA + effet coûts&levier op. = construit
- CA par marque cible vs construit (table + graphe barres natif)
- correction : libellés de total ne commençent plus par "=" (évite #REF)
- 0 erreur, ponts réconciliés

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_CA_v3.xlsx
+++ b/eduservices/EDUSERVICES_Modele_CA_v3.xlsx
@@ -17,6 +17,7 @@
     <sheet name="06_Compta" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="07_PnL" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="08_Saisie_Campus" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="09_Reporting" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,7 +31,7 @@
     <numFmt numFmtId="165" formatCode="#,##0&quot; €&quot;;(#,##0)&quot; €&quot;;&quot;-&quot;"/>
     <numFmt numFmtId="166" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,6 +85,12 @@
       <name val="Arial"/>
       <color rgb="000000FF"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="16"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -123,7 +130,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -145,11 +152,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -315,6 +366,29 @@
     <xf numFmtId="165" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -389,6 +463,140 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>CA par marque — cible vs construit</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'09_Reporting'!G11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'09_Reporting'!$F$12:$F$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'09_Reporting'!$G$12:$G$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'09_Reporting'!H11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'09_Reporting'!$F$12:$F$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'09_Reporting'!$H$12:$H$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1297,6 +1505,406 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:N23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="3" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="2" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>REPORTING — impact live du cadrage · pont d'explication CA &amp; EBITDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="59">
+        <f>'04_Moteur'!$AA$62</f>
+        <v/>
+      </c>
+      <c r="C3" s="60" t="n"/>
+      <c r="D3" s="61" t="n"/>
+      <c r="E3" s="59">
+        <f>'07_PnL'!$G$33</f>
+        <v/>
+      </c>
+      <c r="F3" s="60" t="n"/>
+      <c r="G3" s="61" t="n"/>
+      <c r="H3" s="62">
+        <f>IFERROR('07_PnL'!$G$33/'04_Moteur'!$AA$62,0)</f>
+        <v/>
+      </c>
+      <c r="I3" s="60" t="n"/>
+      <c r="J3" s="61" t="n"/>
+      <c r="K3" s="63">
+        <f>'04_Moteur'!$Y$62</f>
+        <v/>
+      </c>
+      <c r="L3" s="60" t="n"/>
+      <c r="M3" s="61" t="n"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="64" t="inlineStr">
+        <is>
+          <t>CA construit (budget)</t>
+        </is>
+      </c>
+      <c r="C4" s="60" t="n"/>
+      <c r="D4" s="61" t="n"/>
+      <c r="E4" s="64" t="inlineStr">
+        <is>
+          <t>EBITDA construit</t>
+        </is>
+      </c>
+      <c r="F4" s="60" t="n"/>
+      <c r="G4" s="61" t="n"/>
+      <c r="H4" s="65" t="inlineStr">
+        <is>
+          <t>Marge EBITDA</t>
+        </is>
+      </c>
+      <c r="I4" s="60" t="n"/>
+      <c r="J4" s="61" t="n"/>
+      <c r="K4" s="64" t="inlineStr">
+        <is>
+          <t>Effectif construit</t>
+        </is>
+      </c>
+      <c r="L4" s="60" t="n"/>
+      <c r="M4" s="61" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="59">
+        <f>'01_Cadrage'!F7</f>
+        <v/>
+      </c>
+      <c r="C6" s="60" t="n"/>
+      <c r="D6" s="61" t="n"/>
+      <c r="E6" s="66">
+        <f>'01_Cadrage'!D12</f>
+        <v/>
+      </c>
+      <c r="F6" s="60" t="n"/>
+      <c r="G6" s="61" t="n"/>
+      <c r="H6" s="59">
+        <f>IFERROR(SUM('03_Campagnes'!$K$5:$K$18)/SUM('03_Campagnes'!$L$5:$L$18),0)</f>
+        <v/>
+      </c>
+      <c r="I6" s="60" t="n"/>
+      <c r="J6" s="61" t="n"/>
+      <c r="K6" s="59">
+        <f>IFERROR(SUM('03_Campagnes'!$K$5:$K$18)/'04_Moteur'!$W$62,0)</f>
+        <v/>
+      </c>
+      <c r="L6" s="60" t="n"/>
+      <c r="M6" s="61" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="64" t="inlineStr">
+        <is>
+          <t>Écart à la cible CA</t>
+        </is>
+      </c>
+      <c r="C7" s="60" t="n"/>
+      <c r="D7" s="61" t="n"/>
+      <c r="E7" s="67" t="inlineStr">
+        <is>
+          <t>Reste à trouver CA</t>
+        </is>
+      </c>
+      <c r="F7" s="60" t="n"/>
+      <c r="G7" s="61" t="n"/>
+      <c r="H7" s="64" t="inlineStr">
+        <is>
+          <t>CPL effectif moyen</t>
+        </is>
+      </c>
+      <c r="I7" s="60" t="n"/>
+      <c r="J7" s="61" t="n"/>
+      <c r="K7" s="64" t="inlineStr">
+        <is>
+          <t>Coût d'acquisition / inscrit</t>
+        </is>
+      </c>
+      <c r="L7" s="60" t="n"/>
+      <c r="M7" s="61" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Pont CA : Référence 2026 → Budget construit</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="4" t="n"/>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>CA par marque : cible vs construit</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>CA Référence 2026</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="n">
+        <v>21936350</v>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>Marque</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>🎯 Cible</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>🔧 Construit</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>Écart</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="47" t="inlineStr">
+        <is>
+          <t>+ Effet volume</t>
+        </is>
+      </c>
+      <c r="D12" s="15">
+        <f>('04_Moteur'!$Y$62-2952)*(21936350/2952)</f>
+        <v/>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>MBway</t>
+        </is>
+      </c>
+      <c r="G12" s="15">
+        <f>SUMIFS('04_Moteur'!$AJ$4:$AJ$61,'04_Moteur'!$A$4:$A$61,F12)</f>
+        <v/>
+      </c>
+      <c r="H12" s="14">
+        <f>SUMIFS('04_Moteur'!$AA$4:$AA$61,'04_Moteur'!$A$4:$A$61,F12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="15">
+        <f>H12-G12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="47" t="inlineStr">
+        <is>
+          <t>+ Effet prix &amp; mix</t>
+        </is>
+      </c>
+      <c r="D13" s="15">
+        <f>'04_Moteur'!$AA$62-21936350-D12</f>
+        <v/>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>ISCOM</t>
+        </is>
+      </c>
+      <c r="G13" s="15">
+        <f>SUMIFS('04_Moteur'!$AJ$4:$AJ$61,'04_Moteur'!$A$4:$A$61,F13)</f>
+        <v/>
+      </c>
+      <c r="H13" s="14">
+        <f>SUMIFS('04_Moteur'!$AA$4:$AA$61,'04_Moteur'!$A$4:$A$61,F13)</f>
+        <v/>
+      </c>
+      <c r="I13" s="15">
+        <f>H13-G13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="41" t="inlineStr">
+        <is>
+          <t>→ CA Budget construit</t>
+        </is>
+      </c>
+      <c r="D14" s="44">
+        <f>'04_Moteur'!$AA$62</f>
+        <v/>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>Ipac Bachelor Factory</t>
+        </is>
+      </c>
+      <c r="G14" s="15">
+        <f>SUMIFS('04_Moteur'!$AJ$4:$AJ$61,'04_Moteur'!$A$4:$A$61,F14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="14">
+        <f>SUMIFS('04_Moteur'!$AA$4:$AA$61,'04_Moteur'!$A$4:$A$61,F14)</f>
+        <v/>
+      </c>
+      <c r="I14" s="15">
+        <f>H14-G14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="F15" s="17" t="inlineStr">
+        <is>
+          <t>Pigier</t>
+        </is>
+      </c>
+      <c r="G15" s="15">
+        <f>SUMIFS('04_Moteur'!$AJ$4:$AJ$61,'04_Moteur'!$A$4:$A$61,F15)</f>
+        <v/>
+      </c>
+      <c r="H15" s="14">
+        <f>SUMIFS('04_Moteur'!$AA$4:$AA$61,'04_Moteur'!$A$4:$A$61,F15)</f>
+        <v/>
+      </c>
+      <c r="I15" s="15">
+        <f>H15-G15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Pont EBITDA : Référence 2026 → Budget construit</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+      <c r="F16" s="17" t="inlineStr">
+        <is>
+          <t>Tunon</t>
+        </is>
+      </c>
+      <c r="G16" s="15">
+        <f>SUMIFS('04_Moteur'!$AJ$4:$AJ$61,'04_Moteur'!$A$4:$A$61,F16)</f>
+        <v/>
+      </c>
+      <c r="H16" s="14">
+        <f>SUMIFS('04_Moteur'!$AA$4:$AA$61,'04_Moteur'!$A$4:$A$61,F16)</f>
+        <v/>
+      </c>
+      <c r="I16" s="15">
+        <f>H16-G16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>EBITDA Référence 2026</t>
+        </is>
+      </c>
+      <c r="D17" s="13">
+        <f>'07_PnL'!$F$33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="47" t="inlineStr">
+        <is>
+          <t>+ Effet CA (à marge réf.)</t>
+        </is>
+      </c>
+      <c r="D18" s="15">
+        <f>('04_Moteur'!$AA$62-21936350)*IFERROR('07_PnL'!$F$33/21936350,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="47" t="inlineStr">
+        <is>
+          <t>+ Effet coûts &amp; levier op.</t>
+        </is>
+      </c>
+      <c r="D19" s="15">
+        <f>'07_PnL'!$G$33-'07_PnL'!$F$33-D18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="41" t="inlineStr">
+        <is>
+          <t>→ EBITDA Budget construit</t>
+        </is>
+      </c>
+      <c r="D20" s="44">
+        <f>'07_PnL'!$G$33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="32" t="inlineStr">
+        <is>
+          <t>Les tuiles et les ponts se recalculent en direct quand on bouge un levier du cadrage ou un scénario.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="K7:M7"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="K4:M4"/>
+    <mergeCell ref="K6:M6"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B23:N23"/>
+    <mergeCell ref="B1:N1"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="H6:J6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Allocation en cascade groupe → campus avec clé au choix (EBITDA pleinement chargé)
- 10_Allocation : les coûts du siège (3,47 M€) redescendent sur les campus par
  une CLÉ SÉLECTIONNABLE (CA / effectif / nombre de classes)
- par campus : CA → contribution → coûts propres → quote-part groupe →
  EBITDA pleinement chargé + marge %, échelle de couleur (rentable/déficitaire)
- tie-out : Σ EBITDA campus = EBITDA groupe (3 202 713 €), invariant quelle que
  soit la clé — seule la répartition change (effet « piège »)
- 0 erreur

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_CA_v3.xlsx
+++ b/eduservices/EDUSERVICES_Modele_CA_v3.xlsx
@@ -18,6 +18,7 @@
     <sheet name="07_PnL" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="08_Saisie_Campus" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="09_Reporting" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="10_Allocation" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1905,6 +1906,868 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ALLOCATION EN CASCADE — coûts du siège redescendus sur les campus (clé au choix)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Clé d'allocation des coûts groupe :</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>Chiffre d'affaires</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Coûts groupe à répartir :</t>
+        </is>
+      </c>
+      <c r="I3" s="14">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$A$4:$A$675,"GROUPE",'06_Compta'!$H$4:$H$675,"Charge",'06_Compta'!$J$4:$J$675,"2026ATT_VDEF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Marque</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Ville</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Coûts directs</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Contribution</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>Coûts propres campus</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>Clé</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>Quote-part groupe</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>EBITDA campus</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>Marge %</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>MBway</t>
+        </is>
+      </c>
+      <c r="B6" s="39" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="C6" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A6,'06_Compta'!$D$4:$D$675,B6,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Produit")</f>
+        <v/>
+      </c>
+      <c r="D6" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A6,'06_Compta'!$D$4:$D$675,B6,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Coûts directs")</f>
+        <v/>
+      </c>
+      <c r="E6" s="15">
+        <f>C6-D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A6,'06_Compta'!$D$4:$D$675,B6,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Charge")-D6-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A6,'06_Compta'!$D$4:$D$675,B6,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Dotations")</f>
+        <v/>
+      </c>
+      <c r="G6" s="23">
+        <f>IF($E$3="Effectif",SUMIFS('02_Base'!$M$4:$M$61,'02_Base'!$A$4:$A$61,A6,'02_Base'!$B$4:$B$61,B6),IF($E$3="Nombre de classes",SUMIFS('02_Base'!$O$4:$O$61,'02_Base'!$A$4:$A$61,A6,'02_Base'!$B$4:$B$61,B6),C6))</f>
+        <v/>
+      </c>
+      <c r="H6" s="25">
+        <f>IFERROR(G6/SUM($G$6:$G$19),0)</f>
+        <v/>
+      </c>
+      <c r="I6" s="15">
+        <f>H6*$I$3</f>
+        <v/>
+      </c>
+      <c r="J6" s="14">
+        <f>E6-F6-I6</f>
+        <v/>
+      </c>
+      <c r="K6" s="16">
+        <f>IFERROR(J6/C6,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>MBway</t>
+        </is>
+      </c>
+      <c r="B7" s="39" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="C7" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A7,'06_Compta'!$D$4:$D$675,B7,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Produit")</f>
+        <v/>
+      </c>
+      <c r="D7" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A7,'06_Compta'!$D$4:$D$675,B7,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Coûts directs")</f>
+        <v/>
+      </c>
+      <c r="E7" s="15">
+        <f>C7-D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A7,'06_Compta'!$D$4:$D$675,B7,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Charge")-D7-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A7,'06_Compta'!$D$4:$D$675,B7,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Dotations")</f>
+        <v/>
+      </c>
+      <c r="G7" s="23">
+        <f>IF($E$3="Effectif",SUMIFS('02_Base'!$M$4:$M$61,'02_Base'!$A$4:$A$61,A7,'02_Base'!$B$4:$B$61,B7),IF($E$3="Nombre de classes",SUMIFS('02_Base'!$O$4:$O$61,'02_Base'!$A$4:$A$61,A7,'02_Base'!$B$4:$B$61,B7),C7))</f>
+        <v/>
+      </c>
+      <c r="H7" s="25">
+        <f>IFERROR(G7/SUM($G$6:$G$19),0)</f>
+        <v/>
+      </c>
+      <c r="I7" s="15">
+        <f>H7*$I$3</f>
+        <v/>
+      </c>
+      <c r="J7" s="14">
+        <f>E7-F7-I7</f>
+        <v/>
+      </c>
+      <c r="K7" s="16">
+        <f>IFERROR(J7/C7,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>MBway</t>
+        </is>
+      </c>
+      <c r="B8" s="39" t="inlineStr">
+        <is>
+          <t>Nantes</t>
+        </is>
+      </c>
+      <c r="C8" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A8,'06_Compta'!$D$4:$D$675,B8,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Produit")</f>
+        <v/>
+      </c>
+      <c r="D8" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A8,'06_Compta'!$D$4:$D$675,B8,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Coûts directs")</f>
+        <v/>
+      </c>
+      <c r="E8" s="15">
+        <f>C8-D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A8,'06_Compta'!$D$4:$D$675,B8,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Charge")-D8-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A8,'06_Compta'!$D$4:$D$675,B8,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Dotations")</f>
+        <v/>
+      </c>
+      <c r="G8" s="23">
+        <f>IF($E$3="Effectif",SUMIFS('02_Base'!$M$4:$M$61,'02_Base'!$A$4:$A$61,A8,'02_Base'!$B$4:$B$61,B8),IF($E$3="Nombre de classes",SUMIFS('02_Base'!$O$4:$O$61,'02_Base'!$A$4:$A$61,A8,'02_Base'!$B$4:$B$61,B8),C8))</f>
+        <v/>
+      </c>
+      <c r="H8" s="25">
+        <f>IFERROR(G8/SUM($G$6:$G$19),0)</f>
+        <v/>
+      </c>
+      <c r="I8" s="15">
+        <f>H8*$I$3</f>
+        <v/>
+      </c>
+      <c r="J8" s="14">
+        <f>E8-F8-I8</f>
+        <v/>
+      </c>
+      <c r="K8" s="16">
+        <f>IFERROR(J8/C8,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>MBway</t>
+        </is>
+      </c>
+      <c r="B9" s="39" t="inlineStr">
+        <is>
+          <t>Bordeaux</t>
+        </is>
+      </c>
+      <c r="C9" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A9,'06_Compta'!$D$4:$D$675,B9,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Produit")</f>
+        <v/>
+      </c>
+      <c r="D9" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A9,'06_Compta'!$D$4:$D$675,B9,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Coûts directs")</f>
+        <v/>
+      </c>
+      <c r="E9" s="15">
+        <f>C9-D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A9,'06_Compta'!$D$4:$D$675,B9,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Charge")-D9-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A9,'06_Compta'!$D$4:$D$675,B9,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Dotations")</f>
+        <v/>
+      </c>
+      <c r="G9" s="23">
+        <f>IF($E$3="Effectif",SUMIFS('02_Base'!$M$4:$M$61,'02_Base'!$A$4:$A$61,A9,'02_Base'!$B$4:$B$61,B9),IF($E$3="Nombre de classes",SUMIFS('02_Base'!$O$4:$O$61,'02_Base'!$A$4:$A$61,A9,'02_Base'!$B$4:$B$61,B9),C9))</f>
+        <v/>
+      </c>
+      <c r="H9" s="25">
+        <f>IFERROR(G9/SUM($G$6:$G$19),0)</f>
+        <v/>
+      </c>
+      <c r="I9" s="15">
+        <f>H9*$I$3</f>
+        <v/>
+      </c>
+      <c r="J9" s="14">
+        <f>E9-F9-I9</f>
+        <v/>
+      </c>
+      <c r="K9" s="16">
+        <f>IFERROR(J9/C9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>ISCOM</t>
+        </is>
+      </c>
+      <c r="B10" s="39" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="C10" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A10,'06_Compta'!$D$4:$D$675,B10,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Produit")</f>
+        <v/>
+      </c>
+      <c r="D10" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A10,'06_Compta'!$D$4:$D$675,B10,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Coûts directs")</f>
+        <v/>
+      </c>
+      <c r="E10" s="15">
+        <f>C10-D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A10,'06_Compta'!$D$4:$D$675,B10,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Charge")-D10-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A10,'06_Compta'!$D$4:$D$675,B10,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Dotations")</f>
+        <v/>
+      </c>
+      <c r="G10" s="23">
+        <f>IF($E$3="Effectif",SUMIFS('02_Base'!$M$4:$M$61,'02_Base'!$A$4:$A$61,A10,'02_Base'!$B$4:$B$61,B10),IF($E$3="Nombre de classes",SUMIFS('02_Base'!$O$4:$O$61,'02_Base'!$A$4:$A$61,A10,'02_Base'!$B$4:$B$61,B10),C10))</f>
+        <v/>
+      </c>
+      <c r="H10" s="25">
+        <f>IFERROR(G10/SUM($G$6:$G$19),0)</f>
+        <v/>
+      </c>
+      <c r="I10" s="15">
+        <f>H10*$I$3</f>
+        <v/>
+      </c>
+      <c r="J10" s="14">
+        <f>E10-F10-I10</f>
+        <v/>
+      </c>
+      <c r="K10" s="16">
+        <f>IFERROR(J10/C10,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>ISCOM</t>
+        </is>
+      </c>
+      <c r="B11" s="39" t="inlineStr">
+        <is>
+          <t>Lille</t>
+        </is>
+      </c>
+      <c r="C11" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A11,'06_Compta'!$D$4:$D$675,B11,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Produit")</f>
+        <v/>
+      </c>
+      <c r="D11" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A11,'06_Compta'!$D$4:$D$675,B11,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Coûts directs")</f>
+        <v/>
+      </c>
+      <c r="E11" s="15">
+        <f>C11-D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A11,'06_Compta'!$D$4:$D$675,B11,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Charge")-D11-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A11,'06_Compta'!$D$4:$D$675,B11,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Dotations")</f>
+        <v/>
+      </c>
+      <c r="G11" s="23">
+        <f>IF($E$3="Effectif",SUMIFS('02_Base'!$M$4:$M$61,'02_Base'!$A$4:$A$61,A11,'02_Base'!$B$4:$B$61,B11),IF($E$3="Nombre de classes",SUMIFS('02_Base'!$O$4:$O$61,'02_Base'!$A$4:$A$61,A11,'02_Base'!$B$4:$B$61,B11),C11))</f>
+        <v/>
+      </c>
+      <c r="H11" s="25">
+        <f>IFERROR(G11/SUM($G$6:$G$19),0)</f>
+        <v/>
+      </c>
+      <c r="I11" s="15">
+        <f>H11*$I$3</f>
+        <v/>
+      </c>
+      <c r="J11" s="14">
+        <f>E11-F11-I11</f>
+        <v/>
+      </c>
+      <c r="K11" s="16">
+        <f>IFERROR(J11/C11,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>ISCOM</t>
+        </is>
+      </c>
+      <c r="B12" s="39" t="inlineStr">
+        <is>
+          <t>Toulouse</t>
+        </is>
+      </c>
+      <c r="C12" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A12,'06_Compta'!$D$4:$D$675,B12,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Produit")</f>
+        <v/>
+      </c>
+      <c r="D12" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A12,'06_Compta'!$D$4:$D$675,B12,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Coûts directs")</f>
+        <v/>
+      </c>
+      <c r="E12" s="15">
+        <f>C12-D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A12,'06_Compta'!$D$4:$D$675,B12,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Charge")-D12-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A12,'06_Compta'!$D$4:$D$675,B12,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Dotations")</f>
+        <v/>
+      </c>
+      <c r="G12" s="23">
+        <f>IF($E$3="Effectif",SUMIFS('02_Base'!$M$4:$M$61,'02_Base'!$A$4:$A$61,A12,'02_Base'!$B$4:$B$61,B12),IF($E$3="Nombre de classes",SUMIFS('02_Base'!$O$4:$O$61,'02_Base'!$A$4:$A$61,A12,'02_Base'!$B$4:$B$61,B12),C12))</f>
+        <v/>
+      </c>
+      <c r="H12" s="25">
+        <f>IFERROR(G12/SUM($G$6:$G$19),0)</f>
+        <v/>
+      </c>
+      <c r="I12" s="15">
+        <f>H12*$I$3</f>
+        <v/>
+      </c>
+      <c r="J12" s="14">
+        <f>E12-F12-I12</f>
+        <v/>
+      </c>
+      <c r="K12" s="16">
+        <f>IFERROR(J12/C12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Ipac Bachelor Factory</t>
+        </is>
+      </c>
+      <c r="B13" s="39" t="inlineStr">
+        <is>
+          <t>Nantes</t>
+        </is>
+      </c>
+      <c r="C13" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A13,'06_Compta'!$D$4:$D$675,B13,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Produit")</f>
+        <v/>
+      </c>
+      <c r="D13" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A13,'06_Compta'!$D$4:$D$675,B13,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Coûts directs")</f>
+        <v/>
+      </c>
+      <c r="E13" s="15">
+        <f>C13-D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A13,'06_Compta'!$D$4:$D$675,B13,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Charge")-D13-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A13,'06_Compta'!$D$4:$D$675,B13,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Dotations")</f>
+        <v/>
+      </c>
+      <c r="G13" s="23">
+        <f>IF($E$3="Effectif",SUMIFS('02_Base'!$M$4:$M$61,'02_Base'!$A$4:$A$61,A13,'02_Base'!$B$4:$B$61,B13),IF($E$3="Nombre de classes",SUMIFS('02_Base'!$O$4:$O$61,'02_Base'!$A$4:$A$61,A13,'02_Base'!$B$4:$B$61,B13),C13))</f>
+        <v/>
+      </c>
+      <c r="H13" s="25">
+        <f>IFERROR(G13/SUM($G$6:$G$19),0)</f>
+        <v/>
+      </c>
+      <c r="I13" s="15">
+        <f>H13*$I$3</f>
+        <v/>
+      </c>
+      <c r="J13" s="14">
+        <f>E13-F13-I13</f>
+        <v/>
+      </c>
+      <c r="K13" s="16">
+        <f>IFERROR(J13/C13,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Ipac Bachelor Factory</t>
+        </is>
+      </c>
+      <c r="B14" s="39" t="inlineStr">
+        <is>
+          <t>Rennes</t>
+        </is>
+      </c>
+      <c r="C14" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A14,'06_Compta'!$D$4:$D$675,B14,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Produit")</f>
+        <v/>
+      </c>
+      <c r="D14" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A14,'06_Compta'!$D$4:$D$675,B14,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Coûts directs")</f>
+        <v/>
+      </c>
+      <c r="E14" s="15">
+        <f>C14-D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A14,'06_Compta'!$D$4:$D$675,B14,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Charge")-D14-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A14,'06_Compta'!$D$4:$D$675,B14,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Dotations")</f>
+        <v/>
+      </c>
+      <c r="G14" s="23">
+        <f>IF($E$3="Effectif",SUMIFS('02_Base'!$M$4:$M$61,'02_Base'!$A$4:$A$61,A14,'02_Base'!$B$4:$B$61,B14),IF($E$3="Nombre de classes",SUMIFS('02_Base'!$O$4:$O$61,'02_Base'!$A$4:$A$61,A14,'02_Base'!$B$4:$B$61,B14),C14))</f>
+        <v/>
+      </c>
+      <c r="H14" s="25">
+        <f>IFERROR(G14/SUM($G$6:$G$19),0)</f>
+        <v/>
+      </c>
+      <c r="I14" s="15">
+        <f>H14*$I$3</f>
+        <v/>
+      </c>
+      <c r="J14" s="14">
+        <f>E14-F14-I14</f>
+        <v/>
+      </c>
+      <c r="K14" s="16">
+        <f>IFERROR(J14/C14,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Ipac Bachelor Factory</t>
+        </is>
+      </c>
+      <c r="B15" s="39" t="inlineStr">
+        <is>
+          <t>Montpellier</t>
+        </is>
+      </c>
+      <c r="C15" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A15,'06_Compta'!$D$4:$D$675,B15,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Produit")</f>
+        <v/>
+      </c>
+      <c r="D15" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A15,'06_Compta'!$D$4:$D$675,B15,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Coûts directs")</f>
+        <v/>
+      </c>
+      <c r="E15" s="15">
+        <f>C15-D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A15,'06_Compta'!$D$4:$D$675,B15,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Charge")-D15-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A15,'06_Compta'!$D$4:$D$675,B15,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Dotations")</f>
+        <v/>
+      </c>
+      <c r="G15" s="23">
+        <f>IF($E$3="Effectif",SUMIFS('02_Base'!$M$4:$M$61,'02_Base'!$A$4:$A$61,A15,'02_Base'!$B$4:$B$61,B15),IF($E$3="Nombre de classes",SUMIFS('02_Base'!$O$4:$O$61,'02_Base'!$A$4:$A$61,A15,'02_Base'!$B$4:$B$61,B15),C15))</f>
+        <v/>
+      </c>
+      <c r="H15" s="25">
+        <f>IFERROR(G15/SUM($G$6:$G$19),0)</f>
+        <v/>
+      </c>
+      <c r="I15" s="15">
+        <f>H15*$I$3</f>
+        <v/>
+      </c>
+      <c r="J15" s="14">
+        <f>E15-F15-I15</f>
+        <v/>
+      </c>
+      <c r="K15" s="16">
+        <f>IFERROR(J15/C15,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Pigier</t>
+        </is>
+      </c>
+      <c r="B16" s="39" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="C16" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A16,'06_Compta'!$D$4:$D$675,B16,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Produit")</f>
+        <v/>
+      </c>
+      <c r="D16" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A16,'06_Compta'!$D$4:$D$675,B16,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Coûts directs")</f>
+        <v/>
+      </c>
+      <c r="E16" s="15">
+        <f>C16-D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A16,'06_Compta'!$D$4:$D$675,B16,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Charge")-D16-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A16,'06_Compta'!$D$4:$D$675,B16,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Dotations")</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>IF($E$3="Effectif",SUMIFS('02_Base'!$M$4:$M$61,'02_Base'!$A$4:$A$61,A16,'02_Base'!$B$4:$B$61,B16),IF($E$3="Nombre de classes",SUMIFS('02_Base'!$O$4:$O$61,'02_Base'!$A$4:$A$61,A16,'02_Base'!$B$4:$B$61,B16),C16))</f>
+        <v/>
+      </c>
+      <c r="H16" s="25">
+        <f>IFERROR(G16/SUM($G$6:$G$19),0)</f>
+        <v/>
+      </c>
+      <c r="I16" s="15">
+        <f>H16*$I$3</f>
+        <v/>
+      </c>
+      <c r="J16" s="14">
+        <f>E16-F16-I16</f>
+        <v/>
+      </c>
+      <c r="K16" s="16">
+        <f>IFERROR(J16/C16,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Pigier</t>
+        </is>
+      </c>
+      <c r="B17" s="39" t="inlineStr">
+        <is>
+          <t>Bordeaux</t>
+        </is>
+      </c>
+      <c r="C17" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A17,'06_Compta'!$D$4:$D$675,B17,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Produit")</f>
+        <v/>
+      </c>
+      <c r="D17" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A17,'06_Compta'!$D$4:$D$675,B17,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Coûts directs")</f>
+        <v/>
+      </c>
+      <c r="E17" s="15">
+        <f>C17-D17</f>
+        <v/>
+      </c>
+      <c r="F17" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A17,'06_Compta'!$D$4:$D$675,B17,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Charge")-D17-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A17,'06_Compta'!$D$4:$D$675,B17,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Dotations")</f>
+        <v/>
+      </c>
+      <c r="G17" s="23">
+        <f>IF($E$3="Effectif",SUMIFS('02_Base'!$M$4:$M$61,'02_Base'!$A$4:$A$61,A17,'02_Base'!$B$4:$B$61,B17),IF($E$3="Nombre de classes",SUMIFS('02_Base'!$O$4:$O$61,'02_Base'!$A$4:$A$61,A17,'02_Base'!$B$4:$B$61,B17),C17))</f>
+        <v/>
+      </c>
+      <c r="H17" s="25">
+        <f>IFERROR(G17/SUM($G$6:$G$19),0)</f>
+        <v/>
+      </c>
+      <c r="I17" s="15">
+        <f>H17*$I$3</f>
+        <v/>
+      </c>
+      <c r="J17" s="14">
+        <f>E17-F17-I17</f>
+        <v/>
+      </c>
+      <c r="K17" s="16">
+        <f>IFERROR(J17/C17,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Tunon</t>
+        </is>
+      </c>
+      <c r="B18" s="39" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="C18" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A18,'06_Compta'!$D$4:$D$675,B18,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Produit")</f>
+        <v/>
+      </c>
+      <c r="D18" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A18,'06_Compta'!$D$4:$D$675,B18,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Coûts directs")</f>
+        <v/>
+      </c>
+      <c r="E18" s="15">
+        <f>C18-D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A18,'06_Compta'!$D$4:$D$675,B18,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Charge")-D18-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A18,'06_Compta'!$D$4:$D$675,B18,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Dotations")</f>
+        <v/>
+      </c>
+      <c r="G18" s="23">
+        <f>IF($E$3="Effectif",SUMIFS('02_Base'!$M$4:$M$61,'02_Base'!$A$4:$A$61,A18,'02_Base'!$B$4:$B$61,B18),IF($E$3="Nombre de classes",SUMIFS('02_Base'!$O$4:$O$61,'02_Base'!$A$4:$A$61,A18,'02_Base'!$B$4:$B$61,B18),C18))</f>
+        <v/>
+      </c>
+      <c r="H18" s="25">
+        <f>IFERROR(G18/SUM($G$6:$G$19),0)</f>
+        <v/>
+      </c>
+      <c r="I18" s="15">
+        <f>H18*$I$3</f>
+        <v/>
+      </c>
+      <c r="J18" s="14">
+        <f>E18-F18-I18</f>
+        <v/>
+      </c>
+      <c r="K18" s="16">
+        <f>IFERROR(J18/C18,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Tunon</t>
+        </is>
+      </c>
+      <c r="B19" s="39" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="C19" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A19,'06_Compta'!$D$4:$D$675,B19,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Produit")</f>
+        <v/>
+      </c>
+      <c r="D19" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A19,'06_Compta'!$D$4:$D$675,B19,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Coûts directs")</f>
+        <v/>
+      </c>
+      <c r="E19" s="15">
+        <f>C19-D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="15">
+        <f>SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A19,'06_Compta'!$D$4:$D$675,B19,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$H$4:$H$675,"Charge")-D19-SUMIFS('06_Compta'!$L$4:$L$675,'06_Compta'!$C$4:$C$675,A19,'06_Compta'!$D$4:$D$675,B19,'06_Compta'!$J$4:$J$675,"2026ATT_VDEF",'06_Compta'!$I$4:$I$675,"Dotations")</f>
+        <v/>
+      </c>
+      <c r="G19" s="23">
+        <f>IF($E$3="Effectif",SUMIFS('02_Base'!$M$4:$M$61,'02_Base'!$A$4:$A$61,A19,'02_Base'!$B$4:$B$61,B19),IF($E$3="Nombre de classes",SUMIFS('02_Base'!$O$4:$O$61,'02_Base'!$A$4:$A$61,A19,'02_Base'!$B$4:$B$61,B19),C19))</f>
+        <v/>
+      </c>
+      <c r="H19" s="25">
+        <f>IFERROR(G19/SUM($G$6:$G$19),0)</f>
+        <v/>
+      </c>
+      <c r="I19" s="15">
+        <f>H19*$I$3</f>
+        <v/>
+      </c>
+      <c r="J19" s="14">
+        <f>E19-F19-I19</f>
+        <v/>
+      </c>
+      <c r="K19" s="16">
+        <f>IFERROR(J19/C19,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="41" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B20" s="42" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="C20" s="44">
+        <f>SUM(C6:C19)</f>
+        <v/>
+      </c>
+      <c r="D20" s="44">
+        <f>SUM(D6:D19)</f>
+        <v/>
+      </c>
+      <c r="E20" s="44">
+        <f>SUM(E6:E19)</f>
+        <v/>
+      </c>
+      <c r="F20" s="44">
+        <f>SUM(F6:F19)</f>
+        <v/>
+      </c>
+      <c r="G20" s="43">
+        <f>SUM(G6:G19)</f>
+        <v/>
+      </c>
+      <c r="H20" s="42" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="I20" s="44">
+        <f>SUM(I6:I19)</f>
+        <v/>
+      </c>
+      <c r="J20" s="44">
+        <f>SUM(J6:J19)</f>
+        <v/>
+      </c>
+      <c r="K20" s="55">
+        <f>IFERROR(J20/C20,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="32" t="inlineStr">
+        <is>
+          <t>Change la clé (CA / effectif / classes) → la quote-part du siège se redistribue et l'EBITDA par campus bouge. Un campus rentable en contribution peut devenir déficitaire une fois pleinement chargé (effet « piège »). Le total EBITDA reste constant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A22:K23"/>
+  </mergeCells>
+  <conditionalFormatting sqref="K6:K19">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.14"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="E3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Chiffre d'affaires,Effectif,Nombre de classes"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Renommage « semé » → « cadré (groupe) » + explication des 3 caps proposés
- Terminologie : « semé » remplacé par « cadré (groupe) » (plus clair pour un
  CFO) — masque de saisie (Leads cadrés / Effectif cadré ②), titre et guide
  du moteur, notes. Sens inchangé : valeur pré-allouée top-down avant
  ajustement du contrôleur.
- Lexique (01_Cadrage) : ajout de 4 entrées détaillées — Cap retenu (choix
  CFO), Cap éff. (efficience, CAC bas), Cap mom. (momentum, croissance),
  Cap pot. (potentiel, sous-investissement) + comment lire les 3 ensemble
  (la divergence est le plus instructif).
- Note du bloc cap raccourcie (était clippée) et renvoyée vers le lexique.

Vérifié : 0 erreur ; libellés confirmés dans le fichier.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_CA_v3.xlsx
+++ b/eduservices/EDUSERVICES_Modele_CA_v3.xlsx
@@ -1069,7 +1069,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>Votre périmètre. Vous n'ajustez que vos TAUX OPÉRATIONNELS (🟢 jaune) — prix, budget marketing et cible sont fixés par le groupe. Vos ajustements s'AJOUTENT au semé (ils ne l'écrasent pas) et remontent au modèle en temps réel.</t>
+          <t>Votre périmètre. « Cadrés (groupe) » = valeurs pré-allouées par le groupe (budget marketing, cible) que vous recevez. Vous n'ajustez que vos TAUX OPÉRATIONNELS (🟢 jaune) — prix, budget marketing et cible sont fixés par le groupe. Vos ajustements s'AJOUTENT au cadré (ils ne l'écrasent pas) et remontent au modèle en temps réel.</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Leads semé</t>
+          <t>Leads cadrés (groupe)</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>Effectif semé ②</t>
+          <t>Effectif cadré ② (groupe)</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
@@ -6329,7 +6329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:P80"/>
+  <dimension ref="B1:P84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -6941,7 +6941,7 @@
         <v>0.8100000000000001</v>
       </c>
     </row>
-    <row r="20" ht="40" customHeight="1">
+    <row r="20" ht="30" customHeight="1">
       <c r="B20" s="27" t="inlineStr">
         <is>
           <t>Gain conversion admis → inscrit</t>
@@ -6970,7 +6970,7 @@
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
-          <t>Caps PROPOSÉS (vert) = suggestions mesurées sur l'historique ; le CFO garde la main via « Cap retenu » (bleu). Seuls les caps RELATIFS comptent (la formule normalise). Éff. = efficience (CAC marginal bas) · Mom. = momentum (croissance leads 24→26) · Pot. = potentiel (sous-investissement marketing).</t>
+          <t>Cap retenu (bleu) = choix CFO · Caps proposés (vert) = Éff./Mom./Pot. mesurés sur l'historique. Détail de chacun dans le Lexique (bas de feuille).</t>
         </is>
       </c>
     </row>
@@ -8275,12 +8275,12 @@
     <row r="78" ht="42" customHeight="1">
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>🔵 Cap stratégique</t>
+          <t>🔵 Cap retenu</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Concentre le BUDGET MARKETING d'acquisition sur une marque, à enveloppe groupe CONSTANTE (somme nulle). Monter le cap d'une marque → plus de budget → plus de leads → son CA CONSTRUIT monte, celui des autres baisse. Cap = 1 partout = aucune redistribution.</t>
+          <t>LE choix du CFO. Concentre le BUDGET MARKETING d'acquisition sur une marque, à enveloppe groupe CONSTANTE (somme nulle). Monter le cap d'une marque → plus de budget → plus de leads → son CA CONSTRUIT monte, celui des autres baisse. Cap = 1 partout = aucune redistribution. Seuls les caps RELATIFS comptent (la formule normalise).</t>
         </is>
       </c>
       <c r="D78" s="43" t="n"/>
@@ -8292,12 +8292,12 @@
     <row r="79" ht="42" customHeight="1">
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>Indice prix ville</t>
+          <t>🟢 Cap éff. (proposé)</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>DÉDUIT du réalisé (prix moyen ville ÷ national). Informationnel : la géographie tarifaire est déjà dans les revenus. Non saisissable (sinon double compte).</t>
+          <t>SUGGESTION mesurée : cap ∝ 1 / CAC marginal. Pousse le budget là où l'euro marketing produit le plus d'inscrits (rendement élevé, CAC bas). Le plus rigoureux — tend vers l'allocation qui égalise le CAC marginal entre marques. Cap &gt; 1 = marque efficace, à renforcer.</t>
         </is>
       </c>
       <c r="D79" s="43" t="n"/>
@@ -8309,12 +8309,12 @@
     <row r="80" ht="42" customHeight="1">
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>🔵 Clés d'allocation</t>
+          <t>🟢 Cap mom. (proposé)</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>Le driver de répartition des coûts (CA / effectif / classes), figé par le CFO. Méthode centrale ; les campus ne la choisissent pas, ils contestent l'assiette.</t>
+          <t>SUGGESTION mesurée : cap ∝ taux de croissance des leads 2024→2026. Pousse les marques qui montent déjà. Suit la dynamique commerciale — mais peut sur-investir une marque proche du plafond. Cap &gt; 1 = marque en accélération.</t>
         </is>
       </c>
       <c r="D80" s="43" t="n"/>
@@ -8323,8 +8323,77 @@
       <c r="G80" s="43" t="n"/>
       <c r="H80" s="37" t="n"/>
     </row>
+    <row r="81" ht="42" customHeight="1">
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>🟢 Cap pot. (proposé)</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>SUGGESTION mesurée : cap ∝ 1 / intensité marketing (budget ÷ CA). Pousse les marques SOUS-investies vs leur taille — le potentiel dormant. Plus spéculatif : on parie que la marge de progression existe. Cap &gt; 1 = marque sous-exploitée.</t>
+        </is>
+      </c>
+      <c r="D81" s="43" t="n"/>
+      <c r="E81" s="43" t="n"/>
+      <c r="F81" s="43" t="n"/>
+      <c r="G81" s="43" t="n"/>
+      <c r="H81" s="37" t="n"/>
+    </row>
+    <row r="82" ht="42" customHeight="1">
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Lire les 3 ensemble</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>Le plus instructif est la DIVERGENCE. Ex. une marque avec Éff. et Pot. élevés mais Mom. bas = rentable et sous-exploitée, mais son élan faiblit → au CFO de trancher : je pousse (pari) ou je laisse (prudence) ? Les caps proposés éclairent, ils ne décident pas.</t>
+        </is>
+      </c>
+      <c r="D82" s="43" t="n"/>
+      <c r="E82" s="43" t="n"/>
+      <c r="F82" s="43" t="n"/>
+      <c r="G82" s="43" t="n"/>
+      <c r="H82" s="37" t="n"/>
+    </row>
+    <row r="83" ht="42" customHeight="1">
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Indice prix ville</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>DÉDUIT du réalisé (prix moyen ville ÷ national). Informationnel : la géographie tarifaire est déjà dans les revenus. Non saisissable (sinon double compte).</t>
+        </is>
+      </c>
+      <c r="D83" s="43" t="n"/>
+      <c r="E83" s="43" t="n"/>
+      <c r="F83" s="43" t="n"/>
+      <c r="G83" s="43" t="n"/>
+      <c r="H83" s="37" t="n"/>
+    </row>
+    <row r="84" ht="42" customHeight="1">
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>🔵 Clés d'allocation</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>Le driver de répartition des coûts (CA / effectif / classes), figé par le CFO. Méthode centrale ; les campus ne la choisissent pas, ils contestent l'assiette.</t>
+        </is>
+      </c>
+      <c r="D84" s="43" t="n"/>
+      <c r="E84" s="43" t="n"/>
+      <c r="F84" s="43" t="n"/>
+      <c r="G84" s="43" t="n"/>
+      <c r="H84" s="37" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="38">
+    <mergeCell ref="C84:H84"/>
     <mergeCell ref="J38:K38"/>
     <mergeCell ref="C80:H80"/>
     <mergeCell ref="C75:H75"/>
@@ -8338,9 +8407,11 @@
     <mergeCell ref="J36:K36"/>
     <mergeCell ref="J5:M5"/>
     <mergeCell ref="J32:M33"/>
+    <mergeCell ref="C82:H82"/>
     <mergeCell ref="B31:H31"/>
     <mergeCell ref="C72:H72"/>
     <mergeCell ref="J35:K35"/>
+    <mergeCell ref="C81:H81"/>
     <mergeCell ref="L35:M35"/>
     <mergeCell ref="B27:H27"/>
     <mergeCell ref="B5:G5"/>
@@ -8349,6 +8420,7 @@
     <mergeCell ref="J34:M34"/>
     <mergeCell ref="B70:H70"/>
     <mergeCell ref="C78:H78"/>
+    <mergeCell ref="C83:H83"/>
     <mergeCell ref="C77:H77"/>
     <mergeCell ref="J40:M42"/>
     <mergeCell ref="B14:H14"/>
@@ -16069,7 +16141,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MOTEUR DE CA (cellule) — ① CIBLE (éclatée top-down) · ② CADRÉ (semé) · ③ AJUSTÉ (semé + ajustement contrôleur) · écart</t>
+          <t>MOTEUR DE CA (cellule) — ① CIBLE (éclatée top-down) · ② CADRÉ (groupe) · ③ AJUSTÉ (cadré + ajustement contrôleur) · écart</t>
         </is>
       </c>
     </row>
@@ -25428,7 +25500,7 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>② CADRÉ : le même SANS ajustement (pré-budget semé top-down)</t>
+          <t>② CADRÉ : le même SANS ajustement (pré-budget cadré par le groupe, top-down)</t>
         </is>
       </c>
     </row>
@@ -25440,7 +25512,7 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>🟢 AJUSTEMENTS contrôleur (Δ lead→cand / Δ yield / Δ passage) — s'ajoutent au semé, n'écrasent rien</t>
+          <t>🟢 AJUSTEMENTS contrôleur (Δ lead→cand / Δ yield / Δ passage) — s'ajoutent au cadré, n'écrasent rien</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Socle autonome : frais de dossier en colonne (découplé du cadrage)
Le CA du socle référençait la cellule frais du CADRAGE (décision budget 2027) :
changer les frais du budget déplaçait l'historique 2024/2025 — illogique.

Correctif : les frais de dossier deviennent une COLONNE du socle (« Frais/
inscrit », 90 €, donnée par ligne). Le CA du socle = effectif×revenu +
nouveaux×frais(colonne), entièrement auto-porté, sans dépendance au cadrage.
Le frais du cadrage reste utilisé UNIQUEMENT pour le budget 2027 (moteur).

Les frais restent bien un produit chaque année (droits d'inscription, cpte
708) — donc présents dans le CA de chaque exercice ; ils ne bougent simplement
plus avec un paramètre de budget.

Vérifié : 0 erreur ; socle CA sans référence cadrage ; réconciliation écart 0 ;
EBITDA 14,6 %.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_CA_v3.xlsx
+++ b/eduservices/EDUSERVICES_Modele_CA_v3.xlsx
@@ -8937,7 +8937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V177"/>
+  <dimension ref="A1:W177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -8961,7 +8961,8 @@
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="9" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="9" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -9086,6 +9087,11 @@
       </c>
       <c r="V3" s="11" t="inlineStr">
         <is>
+          <t>Frais/inscrit</t>
+        </is>
+      </c>
+      <c r="W3" s="11" t="inlineStr">
+        <is>
           <t>Exercice</t>
         </is>
       </c>
@@ -9168,10 +9174,13 @@
         <v/>
       </c>
       <c r="U4" s="48">
-        <f>M4*P4+K4*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V4" s="37" t="n">
+        <f>M4*P4+K4*V4</f>
+        <v/>
+      </c>
+      <c r="V4" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W4" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -9253,10 +9262,13 @@
         <v/>
       </c>
       <c r="U5" s="48">
-        <f>M5*P5+K5*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V5" s="37" t="n">
+        <f>M5*P5+K5*V5</f>
+        <v/>
+      </c>
+      <c r="V5" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W5" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -9338,10 +9350,13 @@
         <v/>
       </c>
       <c r="U6" s="48">
-        <f>M6*P6+K6*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V6" s="37" t="n">
+        <f>M6*P6+K6*V6</f>
+        <v/>
+      </c>
+      <c r="V6" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W6" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -9423,10 +9438,13 @@
         <v/>
       </c>
       <c r="U7" s="48">
-        <f>M7*P7+K7*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V7" s="37" t="n">
+        <f>M7*P7+K7*V7</f>
+        <v/>
+      </c>
+      <c r="V7" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W7" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -9508,10 +9526,13 @@
         <v/>
       </c>
       <c r="U8" s="48">
-        <f>M8*P8+K8*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V8" s="37" t="n">
+        <f>M8*P8+K8*V8</f>
+        <v/>
+      </c>
+      <c r="V8" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W8" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -9593,10 +9614,13 @@
         <v/>
       </c>
       <c r="U9" s="48">
-        <f>M9*P9+K9*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V9" s="37" t="n">
+        <f>M9*P9+K9*V9</f>
+        <v/>
+      </c>
+      <c r="V9" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W9" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -9678,10 +9702,13 @@
         <v/>
       </c>
       <c r="U10" s="48">
-        <f>M10*P10+K10*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V10" s="37" t="n">
+        <f>M10*P10+K10*V10</f>
+        <v/>
+      </c>
+      <c r="V10" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W10" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -9763,10 +9790,13 @@
         <v/>
       </c>
       <c r="U11" s="48">
-        <f>M11*P11+K11*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V11" s="37" t="n">
+        <f>M11*P11+K11*V11</f>
+        <v/>
+      </c>
+      <c r="V11" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W11" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -9848,10 +9878,13 @@
         <v/>
       </c>
       <c r="U12" s="48">
-        <f>M12*P12+K12*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V12" s="37" t="n">
+        <f>M12*P12+K12*V12</f>
+        <v/>
+      </c>
+      <c r="V12" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W12" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -9933,10 +9966,13 @@
         <v/>
       </c>
       <c r="U13" s="48">
-        <f>M13*P13+K13*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V13" s="37" t="n">
+        <f>M13*P13+K13*V13</f>
+        <v/>
+      </c>
+      <c r="V13" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W13" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -10018,10 +10054,13 @@
         <v/>
       </c>
       <c r="U14" s="48">
-        <f>M14*P14+K14*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V14" s="37" t="n">
+        <f>M14*P14+K14*V14</f>
+        <v/>
+      </c>
+      <c r="V14" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W14" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -10103,10 +10142,13 @@
         <v/>
       </c>
       <c r="U15" s="48">
-        <f>M15*P15+K15*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V15" s="37" t="n">
+        <f>M15*P15+K15*V15</f>
+        <v/>
+      </c>
+      <c r="V15" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W15" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -10188,10 +10230,13 @@
         <v/>
       </c>
       <c r="U16" s="48">
-        <f>M16*P16+K16*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V16" s="37" t="n">
+        <f>M16*P16+K16*V16</f>
+        <v/>
+      </c>
+      <c r="V16" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W16" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -10273,10 +10318,13 @@
         <v/>
       </c>
       <c r="U17" s="48">
-        <f>M17*P17+K17*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V17" s="37" t="n">
+        <f>M17*P17+K17*V17</f>
+        <v/>
+      </c>
+      <c r="V17" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W17" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -10358,10 +10406,13 @@
         <v/>
       </c>
       <c r="U18" s="48">
-        <f>M18*P18+K18*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V18" s="37" t="n">
+        <f>M18*P18+K18*V18</f>
+        <v/>
+      </c>
+      <c r="V18" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W18" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -10443,10 +10494,13 @@
         <v/>
       </c>
       <c r="U19" s="48">
-        <f>M19*P19+K19*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V19" s="37" t="n">
+        <f>M19*P19+K19*V19</f>
+        <v/>
+      </c>
+      <c r="V19" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W19" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -10528,10 +10582,13 @@
         <v/>
       </c>
       <c r="U20" s="48">
-        <f>M20*P20+K20*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V20" s="37" t="n">
+        <f>M20*P20+K20*V20</f>
+        <v/>
+      </c>
+      <c r="V20" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W20" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -10613,10 +10670,13 @@
         <v/>
       </c>
       <c r="U21" s="48">
-        <f>M21*P21+K21*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V21" s="37" t="n">
+        <f>M21*P21+K21*V21</f>
+        <v/>
+      </c>
+      <c r="V21" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W21" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -10698,10 +10758,13 @@
         <v/>
       </c>
       <c r="U22" s="48">
-        <f>M22*P22+K22*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V22" s="37" t="n">
+        <f>M22*P22+K22*V22</f>
+        <v/>
+      </c>
+      <c r="V22" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W22" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -10783,10 +10846,13 @@
         <v/>
       </c>
       <c r="U23" s="48">
-        <f>M23*P23+K23*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V23" s="37" t="n">
+        <f>M23*P23+K23*V23</f>
+        <v/>
+      </c>
+      <c r="V23" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W23" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -10868,10 +10934,13 @@
         <v/>
       </c>
       <c r="U24" s="48">
-        <f>M24*P24+K24*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V24" s="37" t="n">
+        <f>M24*P24+K24*V24</f>
+        <v/>
+      </c>
+      <c r="V24" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W24" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -10953,10 +11022,13 @@
         <v/>
       </c>
       <c r="U25" s="48">
-        <f>M25*P25+K25*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V25" s="37" t="n">
+        <f>M25*P25+K25*V25</f>
+        <v/>
+      </c>
+      <c r="V25" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W25" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -11038,10 +11110,13 @@
         <v/>
       </c>
       <c r="U26" s="48">
-        <f>M26*P26+K26*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V26" s="37" t="n">
+        <f>M26*P26+K26*V26</f>
+        <v/>
+      </c>
+      <c r="V26" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W26" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -11123,10 +11198,13 @@
         <v/>
       </c>
       <c r="U27" s="48">
-        <f>M27*P27+K27*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V27" s="37" t="n">
+        <f>M27*P27+K27*V27</f>
+        <v/>
+      </c>
+      <c r="V27" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W27" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -11208,10 +11286,13 @@
         <v/>
       </c>
       <c r="U28" s="48">
-        <f>M28*P28+K28*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V28" s="37" t="n">
+        <f>M28*P28+K28*V28</f>
+        <v/>
+      </c>
+      <c r="V28" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W28" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -11293,10 +11374,13 @@
         <v/>
       </c>
       <c r="U29" s="48">
-        <f>M29*P29+K29*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V29" s="37" t="n">
+        <f>M29*P29+K29*V29</f>
+        <v/>
+      </c>
+      <c r="V29" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W29" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -11378,10 +11462,13 @@
         <v/>
       </c>
       <c r="U30" s="48">
-        <f>M30*P30+K30*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V30" s="37" t="n">
+        <f>M30*P30+K30*V30</f>
+        <v/>
+      </c>
+      <c r="V30" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W30" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -11463,10 +11550,13 @@
         <v/>
       </c>
       <c r="U31" s="48">
-        <f>M31*P31+K31*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V31" s="37" t="n">
+        <f>M31*P31+K31*V31</f>
+        <v/>
+      </c>
+      <c r="V31" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W31" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -11548,10 +11638,13 @@
         <v/>
       </c>
       <c r="U32" s="48">
-        <f>M32*P32+K32*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V32" s="37" t="n">
+        <f>M32*P32+K32*V32</f>
+        <v/>
+      </c>
+      <c r="V32" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W32" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -11633,10 +11726,13 @@
         <v/>
       </c>
       <c r="U33" s="48">
-        <f>M33*P33+K33*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V33" s="37" t="n">
+        <f>M33*P33+K33*V33</f>
+        <v/>
+      </c>
+      <c r="V33" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W33" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -11718,10 +11814,13 @@
         <v/>
       </c>
       <c r="U34" s="48">
-        <f>M34*P34+K34*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V34" s="37" t="n">
+        <f>M34*P34+K34*V34</f>
+        <v/>
+      </c>
+      <c r="V34" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W34" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -11803,10 +11902,13 @@
         <v/>
       </c>
       <c r="U35" s="48">
-        <f>M35*P35+K35*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V35" s="37" t="n">
+        <f>M35*P35+K35*V35</f>
+        <v/>
+      </c>
+      <c r="V35" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W35" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -11888,10 +11990,13 @@
         <v/>
       </c>
       <c r="U36" s="48">
-        <f>M36*P36+K36*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V36" s="37" t="n">
+        <f>M36*P36+K36*V36</f>
+        <v/>
+      </c>
+      <c r="V36" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W36" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -11973,10 +12078,13 @@
         <v/>
       </c>
       <c r="U37" s="48">
-        <f>M37*P37+K37*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V37" s="37" t="n">
+        <f>M37*P37+K37*V37</f>
+        <v/>
+      </c>
+      <c r="V37" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W37" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -12058,10 +12166,13 @@
         <v/>
       </c>
       <c r="U38" s="48">
-        <f>M38*P38+K38*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V38" s="37" t="n">
+        <f>M38*P38+K38*V38</f>
+        <v/>
+      </c>
+      <c r="V38" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W38" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -12143,10 +12254,13 @@
         <v/>
       </c>
       <c r="U39" s="48">
-        <f>M39*P39+K39*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V39" s="37" t="n">
+        <f>M39*P39+K39*V39</f>
+        <v/>
+      </c>
+      <c r="V39" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W39" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -12228,10 +12342,13 @@
         <v/>
       </c>
       <c r="U40" s="48">
-        <f>M40*P40+K40*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V40" s="37" t="n">
+        <f>M40*P40+K40*V40</f>
+        <v/>
+      </c>
+      <c r="V40" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W40" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -12313,10 +12430,13 @@
         <v/>
       </c>
       <c r="U41" s="48">
-        <f>M41*P41+K41*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V41" s="37" t="n">
+        <f>M41*P41+K41*V41</f>
+        <v/>
+      </c>
+      <c r="V41" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W41" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -12398,10 +12518,13 @@
         <v/>
       </c>
       <c r="U42" s="48">
-        <f>M42*P42+K42*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V42" s="37" t="n">
+        <f>M42*P42+K42*V42</f>
+        <v/>
+      </c>
+      <c r="V42" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W42" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -12483,10 +12606,13 @@
         <v/>
       </c>
       <c r="U43" s="48">
-        <f>M43*P43+K43*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V43" s="37" t="n">
+        <f>M43*P43+K43*V43</f>
+        <v/>
+      </c>
+      <c r="V43" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W43" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -12568,10 +12694,13 @@
         <v/>
       </c>
       <c r="U44" s="48">
-        <f>M44*P44+K44*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V44" s="37" t="n">
+        <f>M44*P44+K44*V44</f>
+        <v/>
+      </c>
+      <c r="V44" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W44" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -12653,10 +12782,13 @@
         <v/>
       </c>
       <c r="U45" s="48">
-        <f>M45*P45+K45*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V45" s="37" t="n">
+        <f>M45*P45+K45*V45</f>
+        <v/>
+      </c>
+      <c r="V45" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W45" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -12738,10 +12870,13 @@
         <v/>
       </c>
       <c r="U46" s="48">
-        <f>M46*P46+K46*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V46" s="37" t="n">
+        <f>M46*P46+K46*V46</f>
+        <v/>
+      </c>
+      <c r="V46" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W46" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -12823,10 +12958,13 @@
         <v/>
       </c>
       <c r="U47" s="48">
-        <f>M47*P47+K47*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V47" s="37" t="n">
+        <f>M47*P47+K47*V47</f>
+        <v/>
+      </c>
+      <c r="V47" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W47" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -12908,10 +13046,13 @@
         <v/>
       </c>
       <c r="U48" s="48">
-        <f>M48*P48+K48*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V48" s="37" t="n">
+        <f>M48*P48+K48*V48</f>
+        <v/>
+      </c>
+      <c r="V48" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W48" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -12993,10 +13134,13 @@
         <v/>
       </c>
       <c r="U49" s="48">
-        <f>M49*P49+K49*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V49" s="37" t="n">
+        <f>M49*P49+K49*V49</f>
+        <v/>
+      </c>
+      <c r="V49" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W49" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -13078,10 +13222,13 @@
         <v/>
       </c>
       <c r="U50" s="48">
-        <f>M50*P50+K50*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V50" s="37" t="n">
+        <f>M50*P50+K50*V50</f>
+        <v/>
+      </c>
+      <c r="V50" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W50" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -13163,10 +13310,13 @@
         <v/>
       </c>
       <c r="U51" s="48">
-        <f>M51*P51+K51*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V51" s="37" t="n">
+        <f>M51*P51+K51*V51</f>
+        <v/>
+      </c>
+      <c r="V51" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W51" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -13248,10 +13398,13 @@
         <v/>
       </c>
       <c r="U52" s="48">
-        <f>M52*P52+K52*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V52" s="37" t="n">
+        <f>M52*P52+K52*V52</f>
+        <v/>
+      </c>
+      <c r="V52" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W52" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -13333,10 +13486,13 @@
         <v/>
       </c>
       <c r="U53" s="48">
-        <f>M53*P53+K53*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V53" s="37" t="n">
+        <f>M53*P53+K53*V53</f>
+        <v/>
+      </c>
+      <c r="V53" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W53" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -13418,10 +13574,13 @@
         <v/>
       </c>
       <c r="U54" s="48">
-        <f>M54*P54+K54*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V54" s="37" t="n">
+        <f>M54*P54+K54*V54</f>
+        <v/>
+      </c>
+      <c r="V54" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W54" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -13503,10 +13662,13 @@
         <v/>
       </c>
       <c r="U55" s="48">
-        <f>M55*P55+K55*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V55" s="37" t="n">
+        <f>M55*P55+K55*V55</f>
+        <v/>
+      </c>
+      <c r="V55" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W55" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -13588,10 +13750,13 @@
         <v/>
       </c>
       <c r="U56" s="48">
-        <f>M56*P56+K56*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V56" s="37" t="n">
+        <f>M56*P56+K56*V56</f>
+        <v/>
+      </c>
+      <c r="V56" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W56" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -13673,10 +13838,13 @@
         <v/>
       </c>
       <c r="U57" s="48">
-        <f>M57*P57+K57*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V57" s="37" t="n">
+        <f>M57*P57+K57*V57</f>
+        <v/>
+      </c>
+      <c r="V57" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W57" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -13758,10 +13926,13 @@
         <v/>
       </c>
       <c r="U58" s="48">
-        <f>M58*P58+K58*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V58" s="37" t="n">
+        <f>M58*P58+K58*V58</f>
+        <v/>
+      </c>
+      <c r="V58" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W58" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -13843,10 +14014,13 @@
         <v/>
       </c>
       <c r="U59" s="48">
-        <f>M59*P59+K59*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V59" s="37" t="n">
+        <f>M59*P59+K59*V59</f>
+        <v/>
+      </c>
+      <c r="V59" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W59" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -13928,10 +14102,13 @@
         <v/>
       </c>
       <c r="U60" s="48">
-        <f>M60*P60+K60*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V60" s="37" t="n">
+        <f>M60*P60+K60*V60</f>
+        <v/>
+      </c>
+      <c r="V60" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W60" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -14013,10 +14190,13 @@
         <v/>
       </c>
       <c r="U61" s="48">
-        <f>M61*P61+K61*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V61" s="37" t="n">
+        <f>M61*P61+K61*V61</f>
+        <v/>
+      </c>
+      <c r="V61" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W61" s="37" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -14098,10 +14278,13 @@
         <v/>
       </c>
       <c r="U62" s="48">
-        <f>M62*P62+K62*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V62" s="37" t="n">
+        <f>M62*P62+K62*V62</f>
+        <v/>
+      </c>
+      <c r="V62" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W62" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -14183,10 +14366,13 @@
         <v/>
       </c>
       <c r="U63" s="48">
-        <f>M63*P63+K63*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V63" s="37" t="n">
+        <f>M63*P63+K63*V63</f>
+        <v/>
+      </c>
+      <c r="V63" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W63" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -14268,10 +14454,13 @@
         <v/>
       </c>
       <c r="U64" s="48">
-        <f>M64*P64+K64*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V64" s="37" t="n">
+        <f>M64*P64+K64*V64</f>
+        <v/>
+      </c>
+      <c r="V64" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W64" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -14353,10 +14542,13 @@
         <v/>
       </c>
       <c r="U65" s="48">
-        <f>M65*P65+K65*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V65" s="37" t="n">
+        <f>M65*P65+K65*V65</f>
+        <v/>
+      </c>
+      <c r="V65" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W65" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -14438,10 +14630,13 @@
         <v/>
       </c>
       <c r="U66" s="48">
-        <f>M66*P66+K66*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V66" s="37" t="n">
+        <f>M66*P66+K66*V66</f>
+        <v/>
+      </c>
+      <c r="V66" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W66" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -14523,10 +14718,13 @@
         <v/>
       </c>
       <c r="U67" s="48">
-        <f>M67*P67+K67*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V67" s="37" t="n">
+        <f>M67*P67+K67*V67</f>
+        <v/>
+      </c>
+      <c r="V67" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W67" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -14608,10 +14806,13 @@
         <v/>
       </c>
       <c r="U68" s="48">
-        <f>M68*P68+K68*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V68" s="37" t="n">
+        <f>M68*P68+K68*V68</f>
+        <v/>
+      </c>
+      <c r="V68" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W68" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -14693,10 +14894,13 @@
         <v/>
       </c>
       <c r="U69" s="48">
-        <f>M69*P69+K69*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V69" s="37" t="n">
+        <f>M69*P69+K69*V69</f>
+        <v/>
+      </c>
+      <c r="V69" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W69" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -14778,10 +14982,13 @@
         <v/>
       </c>
       <c r="U70" s="48">
-        <f>M70*P70+K70*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V70" s="37" t="n">
+        <f>M70*P70+K70*V70</f>
+        <v/>
+      </c>
+      <c r="V70" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W70" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -14863,10 +15070,13 @@
         <v/>
       </c>
       <c r="U71" s="48">
-        <f>M71*P71+K71*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V71" s="37" t="n">
+        <f>M71*P71+K71*V71</f>
+        <v/>
+      </c>
+      <c r="V71" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W71" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -14948,10 +15158,13 @@
         <v/>
       </c>
       <c r="U72" s="48">
-        <f>M72*P72+K72*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V72" s="37" t="n">
+        <f>M72*P72+K72*V72</f>
+        <v/>
+      </c>
+      <c r="V72" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W72" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -15033,10 +15246,13 @@
         <v/>
       </c>
       <c r="U73" s="48">
-        <f>M73*P73+K73*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V73" s="37" t="n">
+        <f>M73*P73+K73*V73</f>
+        <v/>
+      </c>
+      <c r="V73" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W73" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -15118,10 +15334,13 @@
         <v/>
       </c>
       <c r="U74" s="48">
-        <f>M74*P74+K74*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V74" s="37" t="n">
+        <f>M74*P74+K74*V74</f>
+        <v/>
+      </c>
+      <c r="V74" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W74" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -15203,10 +15422,13 @@
         <v/>
       </c>
       <c r="U75" s="48">
-        <f>M75*P75+K75*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V75" s="37" t="n">
+        <f>M75*P75+K75*V75</f>
+        <v/>
+      </c>
+      <c r="V75" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W75" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -15288,10 +15510,13 @@
         <v/>
       </c>
       <c r="U76" s="48">
-        <f>M76*P76+K76*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V76" s="37" t="n">
+        <f>M76*P76+K76*V76</f>
+        <v/>
+      </c>
+      <c r="V76" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W76" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -15373,10 +15598,13 @@
         <v/>
       </c>
       <c r="U77" s="48">
-        <f>M77*P77+K77*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V77" s="37" t="n">
+        <f>M77*P77+K77*V77</f>
+        <v/>
+      </c>
+      <c r="V77" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W77" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -15458,10 +15686,13 @@
         <v/>
       </c>
       <c r="U78" s="48">
-        <f>M78*P78+K78*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V78" s="37" t="n">
+        <f>M78*P78+K78*V78</f>
+        <v/>
+      </c>
+      <c r="V78" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W78" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -15543,10 +15774,13 @@
         <v/>
       </c>
       <c r="U79" s="48">
-        <f>M79*P79+K79*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V79" s="37" t="n">
+        <f>M79*P79+K79*V79</f>
+        <v/>
+      </c>
+      <c r="V79" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W79" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -15628,10 +15862,13 @@
         <v/>
       </c>
       <c r="U80" s="48">
-        <f>M80*P80+K80*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V80" s="37" t="n">
+        <f>M80*P80+K80*V80</f>
+        <v/>
+      </c>
+      <c r="V80" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W80" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -15713,10 +15950,13 @@
         <v/>
       </c>
       <c r="U81" s="48">
-        <f>M81*P81+K81*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V81" s="37" t="n">
+        <f>M81*P81+K81*V81</f>
+        <v/>
+      </c>
+      <c r="V81" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W81" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -15798,10 +16038,13 @@
         <v/>
       </c>
       <c r="U82" s="48">
-        <f>M82*P82+K82*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V82" s="37" t="n">
+        <f>M82*P82+K82*V82</f>
+        <v/>
+      </c>
+      <c r="V82" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W82" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -15883,10 +16126,13 @@
         <v/>
       </c>
       <c r="U83" s="48">
-        <f>M83*P83+K83*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V83" s="37" t="n">
+        <f>M83*P83+K83*V83</f>
+        <v/>
+      </c>
+      <c r="V83" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W83" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -15968,10 +16214,13 @@
         <v/>
       </c>
       <c r="U84" s="48">
-        <f>M84*P84+K84*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V84" s="37" t="n">
+        <f>M84*P84+K84*V84</f>
+        <v/>
+      </c>
+      <c r="V84" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W84" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -16053,10 +16302,13 @@
         <v/>
       </c>
       <c r="U85" s="48">
-        <f>M85*P85+K85*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V85" s="37" t="n">
+        <f>M85*P85+K85*V85</f>
+        <v/>
+      </c>
+      <c r="V85" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W85" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -16138,10 +16390,13 @@
         <v/>
       </c>
       <c r="U86" s="48">
-        <f>M86*P86+K86*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V86" s="37" t="n">
+        <f>M86*P86+K86*V86</f>
+        <v/>
+      </c>
+      <c r="V86" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W86" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -16223,10 +16478,13 @@
         <v/>
       </c>
       <c r="U87" s="48">
-        <f>M87*P87+K87*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V87" s="37" t="n">
+        <f>M87*P87+K87*V87</f>
+        <v/>
+      </c>
+      <c r="V87" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W87" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -16308,10 +16566,13 @@
         <v/>
       </c>
       <c r="U88" s="48">
-        <f>M88*P88+K88*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V88" s="37" t="n">
+        <f>M88*P88+K88*V88</f>
+        <v/>
+      </c>
+      <c r="V88" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W88" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -16393,10 +16654,13 @@
         <v/>
       </c>
       <c r="U89" s="48">
-        <f>M89*P89+K89*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V89" s="37" t="n">
+        <f>M89*P89+K89*V89</f>
+        <v/>
+      </c>
+      <c r="V89" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W89" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -16478,10 +16742,13 @@
         <v/>
       </c>
       <c r="U90" s="48">
-        <f>M90*P90+K90*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V90" s="37" t="n">
+        <f>M90*P90+K90*V90</f>
+        <v/>
+      </c>
+      <c r="V90" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W90" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -16563,10 +16830,13 @@
         <v/>
       </c>
       <c r="U91" s="48">
-        <f>M91*P91+K91*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V91" s="37" t="n">
+        <f>M91*P91+K91*V91</f>
+        <v/>
+      </c>
+      <c r="V91" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W91" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -16648,10 +16918,13 @@
         <v/>
       </c>
       <c r="U92" s="48">
-        <f>M92*P92+K92*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V92" s="37" t="n">
+        <f>M92*P92+K92*V92</f>
+        <v/>
+      </c>
+      <c r="V92" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W92" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -16733,10 +17006,13 @@
         <v/>
       </c>
       <c r="U93" s="48">
-        <f>M93*P93+K93*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V93" s="37" t="n">
+        <f>M93*P93+K93*V93</f>
+        <v/>
+      </c>
+      <c r="V93" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W93" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -16818,10 +17094,13 @@
         <v/>
       </c>
       <c r="U94" s="48">
-        <f>M94*P94+K94*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V94" s="37" t="n">
+        <f>M94*P94+K94*V94</f>
+        <v/>
+      </c>
+      <c r="V94" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W94" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -16903,10 +17182,13 @@
         <v/>
       </c>
       <c r="U95" s="48">
-        <f>M95*P95+K95*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V95" s="37" t="n">
+        <f>M95*P95+K95*V95</f>
+        <v/>
+      </c>
+      <c r="V95" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W95" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -16988,10 +17270,13 @@
         <v/>
       </c>
       <c r="U96" s="48">
-        <f>M96*P96+K96*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V96" s="37" t="n">
+        <f>M96*P96+K96*V96</f>
+        <v/>
+      </c>
+      <c r="V96" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W96" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -17073,10 +17358,13 @@
         <v/>
       </c>
       <c r="U97" s="48">
-        <f>M97*P97+K97*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V97" s="37" t="n">
+        <f>M97*P97+K97*V97</f>
+        <v/>
+      </c>
+      <c r="V97" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W97" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -17158,10 +17446,13 @@
         <v/>
       </c>
       <c r="U98" s="48">
-        <f>M98*P98+K98*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V98" s="37" t="n">
+        <f>M98*P98+K98*V98</f>
+        <v/>
+      </c>
+      <c r="V98" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W98" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -17243,10 +17534,13 @@
         <v/>
       </c>
       <c r="U99" s="48">
-        <f>M99*P99+K99*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V99" s="37" t="n">
+        <f>M99*P99+K99*V99</f>
+        <v/>
+      </c>
+      <c r="V99" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W99" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -17328,10 +17622,13 @@
         <v/>
       </c>
       <c r="U100" s="48">
-        <f>M100*P100+K100*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V100" s="37" t="n">
+        <f>M100*P100+K100*V100</f>
+        <v/>
+      </c>
+      <c r="V100" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W100" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -17413,10 +17710,13 @@
         <v/>
       </c>
       <c r="U101" s="48">
-        <f>M101*P101+K101*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V101" s="37" t="n">
+        <f>M101*P101+K101*V101</f>
+        <v/>
+      </c>
+      <c r="V101" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W101" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -17498,10 +17798,13 @@
         <v/>
       </c>
       <c r="U102" s="48">
-        <f>M102*P102+K102*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V102" s="37" t="n">
+        <f>M102*P102+K102*V102</f>
+        <v/>
+      </c>
+      <c r="V102" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W102" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -17583,10 +17886,13 @@
         <v/>
       </c>
       <c r="U103" s="48">
-        <f>M103*P103+K103*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V103" s="37" t="n">
+        <f>M103*P103+K103*V103</f>
+        <v/>
+      </c>
+      <c r="V103" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W103" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -17668,10 +17974,13 @@
         <v/>
       </c>
       <c r="U104" s="48">
-        <f>M104*P104+K104*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V104" s="37" t="n">
+        <f>M104*P104+K104*V104</f>
+        <v/>
+      </c>
+      <c r="V104" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W104" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -17753,10 +18062,13 @@
         <v/>
       </c>
       <c r="U105" s="48">
-        <f>M105*P105+K105*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V105" s="37" t="n">
+        <f>M105*P105+K105*V105</f>
+        <v/>
+      </c>
+      <c r="V105" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W105" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -17838,10 +18150,13 @@
         <v/>
       </c>
       <c r="U106" s="48">
-        <f>M106*P106+K106*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V106" s="37" t="n">
+        <f>M106*P106+K106*V106</f>
+        <v/>
+      </c>
+      <c r="V106" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W106" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -17923,10 +18238,13 @@
         <v/>
       </c>
       <c r="U107" s="48">
-        <f>M107*P107+K107*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V107" s="37" t="n">
+        <f>M107*P107+K107*V107</f>
+        <v/>
+      </c>
+      <c r="V107" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W107" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -18008,10 +18326,13 @@
         <v/>
       </c>
       <c r="U108" s="48">
-        <f>M108*P108+K108*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V108" s="37" t="n">
+        <f>M108*P108+K108*V108</f>
+        <v/>
+      </c>
+      <c r="V108" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W108" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -18093,10 +18414,13 @@
         <v/>
       </c>
       <c r="U109" s="48">
-        <f>M109*P109+K109*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V109" s="37" t="n">
+        <f>M109*P109+K109*V109</f>
+        <v/>
+      </c>
+      <c r="V109" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W109" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -18178,10 +18502,13 @@
         <v/>
       </c>
       <c r="U110" s="48">
-        <f>M110*P110+K110*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V110" s="37" t="n">
+        <f>M110*P110+K110*V110</f>
+        <v/>
+      </c>
+      <c r="V110" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W110" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -18263,10 +18590,13 @@
         <v/>
       </c>
       <c r="U111" s="48">
-        <f>M111*P111+K111*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V111" s="37" t="n">
+        <f>M111*P111+K111*V111</f>
+        <v/>
+      </c>
+      <c r="V111" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W111" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -18348,10 +18678,13 @@
         <v/>
       </c>
       <c r="U112" s="48">
-        <f>M112*P112+K112*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V112" s="37" t="n">
+        <f>M112*P112+K112*V112</f>
+        <v/>
+      </c>
+      <c r="V112" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W112" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -18433,10 +18766,13 @@
         <v/>
       </c>
       <c r="U113" s="48">
-        <f>M113*P113+K113*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V113" s="37" t="n">
+        <f>M113*P113+K113*V113</f>
+        <v/>
+      </c>
+      <c r="V113" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W113" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -18518,10 +18854,13 @@
         <v/>
       </c>
       <c r="U114" s="48">
-        <f>M114*P114+K114*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V114" s="37" t="n">
+        <f>M114*P114+K114*V114</f>
+        <v/>
+      </c>
+      <c r="V114" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W114" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -18603,10 +18942,13 @@
         <v/>
       </c>
       <c r="U115" s="48">
-        <f>M115*P115+K115*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V115" s="37" t="n">
+        <f>M115*P115+K115*V115</f>
+        <v/>
+      </c>
+      <c r="V115" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W115" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -18688,10 +19030,13 @@
         <v/>
       </c>
       <c r="U116" s="48">
-        <f>M116*P116+K116*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V116" s="37" t="n">
+        <f>M116*P116+K116*V116</f>
+        <v/>
+      </c>
+      <c r="V116" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W116" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -18773,10 +19118,13 @@
         <v/>
       </c>
       <c r="U117" s="48">
-        <f>M117*P117+K117*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V117" s="37" t="n">
+        <f>M117*P117+K117*V117</f>
+        <v/>
+      </c>
+      <c r="V117" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W117" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -18858,10 +19206,13 @@
         <v/>
       </c>
       <c r="U118" s="48">
-        <f>M118*P118+K118*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V118" s="37" t="n">
+        <f>M118*P118+K118*V118</f>
+        <v/>
+      </c>
+      <c r="V118" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W118" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -18943,10 +19294,13 @@
         <v/>
       </c>
       <c r="U119" s="48">
-        <f>M119*P119+K119*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V119" s="37" t="n">
+        <f>M119*P119+K119*V119</f>
+        <v/>
+      </c>
+      <c r="V119" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W119" s="37" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -19028,10 +19382,13 @@
         <v/>
       </c>
       <c r="U120" s="48">
-        <f>M120*P120+K120*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V120" s="37" t="n">
+        <f>M120*P120+K120*V120</f>
+        <v/>
+      </c>
+      <c r="V120" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W120" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -19113,10 +19470,13 @@
         <v/>
       </c>
       <c r="U121" s="48">
-        <f>M121*P121+K121*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V121" s="37" t="n">
+        <f>M121*P121+K121*V121</f>
+        <v/>
+      </c>
+      <c r="V121" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W121" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -19198,10 +19558,13 @@
         <v/>
       </c>
       <c r="U122" s="48">
-        <f>M122*P122+K122*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V122" s="37" t="n">
+        <f>M122*P122+K122*V122</f>
+        <v/>
+      </c>
+      <c r="V122" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W122" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -19283,10 +19646,13 @@
         <v/>
       </c>
       <c r="U123" s="48">
-        <f>M123*P123+K123*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V123" s="37" t="n">
+        <f>M123*P123+K123*V123</f>
+        <v/>
+      </c>
+      <c r="V123" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W123" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -19368,10 +19734,13 @@
         <v/>
       </c>
       <c r="U124" s="48">
-        <f>M124*P124+K124*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V124" s="37" t="n">
+        <f>M124*P124+K124*V124</f>
+        <v/>
+      </c>
+      <c r="V124" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W124" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -19453,10 +19822,13 @@
         <v/>
       </c>
       <c r="U125" s="48">
-        <f>M125*P125+K125*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V125" s="37" t="n">
+        <f>M125*P125+K125*V125</f>
+        <v/>
+      </c>
+      <c r="V125" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W125" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -19538,10 +19910,13 @@
         <v/>
       </c>
       <c r="U126" s="48">
-        <f>M126*P126+K126*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V126" s="37" t="n">
+        <f>M126*P126+K126*V126</f>
+        <v/>
+      </c>
+      <c r="V126" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W126" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -19623,10 +19998,13 @@
         <v/>
       </c>
       <c r="U127" s="48">
-        <f>M127*P127+K127*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V127" s="37" t="n">
+        <f>M127*P127+K127*V127</f>
+        <v/>
+      </c>
+      <c r="V127" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W127" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -19708,10 +20086,13 @@
         <v/>
       </c>
       <c r="U128" s="48">
-        <f>M128*P128+K128*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V128" s="37" t="n">
+        <f>M128*P128+K128*V128</f>
+        <v/>
+      </c>
+      <c r="V128" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W128" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -19793,10 +20174,13 @@
         <v/>
       </c>
       <c r="U129" s="48">
-        <f>M129*P129+K129*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V129" s="37" t="n">
+        <f>M129*P129+K129*V129</f>
+        <v/>
+      </c>
+      <c r="V129" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W129" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -19878,10 +20262,13 @@
         <v/>
       </c>
       <c r="U130" s="48">
-        <f>M130*P130+K130*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V130" s="37" t="n">
+        <f>M130*P130+K130*V130</f>
+        <v/>
+      </c>
+      <c r="V130" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W130" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -19963,10 +20350,13 @@
         <v/>
       </c>
       <c r="U131" s="48">
-        <f>M131*P131+K131*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V131" s="37" t="n">
+        <f>M131*P131+K131*V131</f>
+        <v/>
+      </c>
+      <c r="V131" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W131" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -20048,10 +20438,13 @@
         <v/>
       </c>
       <c r="U132" s="48">
-        <f>M132*P132+K132*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V132" s="37" t="n">
+        <f>M132*P132+K132*V132</f>
+        <v/>
+      </c>
+      <c r="V132" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W132" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -20133,10 +20526,13 @@
         <v/>
       </c>
       <c r="U133" s="48">
-        <f>M133*P133+K133*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V133" s="37" t="n">
+        <f>M133*P133+K133*V133</f>
+        <v/>
+      </c>
+      <c r="V133" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W133" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -20218,10 +20614,13 @@
         <v/>
       </c>
       <c r="U134" s="48">
-        <f>M134*P134+K134*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V134" s="37" t="n">
+        <f>M134*P134+K134*V134</f>
+        <v/>
+      </c>
+      <c r="V134" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W134" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -20303,10 +20702,13 @@
         <v/>
       </c>
       <c r="U135" s="48">
-        <f>M135*P135+K135*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V135" s="37" t="n">
+        <f>M135*P135+K135*V135</f>
+        <v/>
+      </c>
+      <c r="V135" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W135" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -20388,10 +20790,13 @@
         <v/>
       </c>
       <c r="U136" s="48">
-        <f>M136*P136+K136*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V136" s="37" t="n">
+        <f>M136*P136+K136*V136</f>
+        <v/>
+      </c>
+      <c r="V136" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W136" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -20473,10 +20878,13 @@
         <v/>
       </c>
       <c r="U137" s="48">
-        <f>M137*P137+K137*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V137" s="37" t="n">
+        <f>M137*P137+K137*V137</f>
+        <v/>
+      </c>
+      <c r="V137" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W137" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -20558,10 +20966,13 @@
         <v/>
       </c>
       <c r="U138" s="48">
-        <f>M138*P138+K138*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V138" s="37" t="n">
+        <f>M138*P138+K138*V138</f>
+        <v/>
+      </c>
+      <c r="V138" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W138" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -20643,10 +21054,13 @@
         <v/>
       </c>
       <c r="U139" s="48">
-        <f>M139*P139+K139*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V139" s="37" t="n">
+        <f>M139*P139+K139*V139</f>
+        <v/>
+      </c>
+      <c r="V139" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W139" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -20728,10 +21142,13 @@
         <v/>
       </c>
       <c r="U140" s="48">
-        <f>M140*P140+K140*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V140" s="37" t="n">
+        <f>M140*P140+K140*V140</f>
+        <v/>
+      </c>
+      <c r="V140" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W140" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -20813,10 +21230,13 @@
         <v/>
       </c>
       <c r="U141" s="48">
-        <f>M141*P141+K141*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V141" s="37" t="n">
+        <f>M141*P141+K141*V141</f>
+        <v/>
+      </c>
+      <c r="V141" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W141" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -20898,10 +21318,13 @@
         <v/>
       </c>
       <c r="U142" s="48">
-        <f>M142*P142+K142*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V142" s="37" t="n">
+        <f>M142*P142+K142*V142</f>
+        <v/>
+      </c>
+      <c r="V142" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W142" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -20983,10 +21406,13 @@
         <v/>
       </c>
       <c r="U143" s="48">
-        <f>M143*P143+K143*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V143" s="37" t="n">
+        <f>M143*P143+K143*V143</f>
+        <v/>
+      </c>
+      <c r="V143" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W143" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -21068,10 +21494,13 @@
         <v/>
       </c>
       <c r="U144" s="48">
-        <f>M144*P144+K144*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V144" s="37" t="n">
+        <f>M144*P144+K144*V144</f>
+        <v/>
+      </c>
+      <c r="V144" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W144" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -21153,10 +21582,13 @@
         <v/>
       </c>
       <c r="U145" s="48">
-        <f>M145*P145+K145*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V145" s="37" t="n">
+        <f>M145*P145+K145*V145</f>
+        <v/>
+      </c>
+      <c r="V145" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W145" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -21238,10 +21670,13 @@
         <v/>
       </c>
       <c r="U146" s="48">
-        <f>M146*P146+K146*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V146" s="37" t="n">
+        <f>M146*P146+K146*V146</f>
+        <v/>
+      </c>
+      <c r="V146" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W146" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -21323,10 +21758,13 @@
         <v/>
       </c>
       <c r="U147" s="48">
-        <f>M147*P147+K147*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V147" s="37" t="n">
+        <f>M147*P147+K147*V147</f>
+        <v/>
+      </c>
+      <c r="V147" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W147" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -21408,10 +21846,13 @@
         <v/>
       </c>
       <c r="U148" s="48">
-        <f>M148*P148+K148*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V148" s="37" t="n">
+        <f>M148*P148+K148*V148</f>
+        <v/>
+      </c>
+      <c r="V148" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W148" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -21493,10 +21934,13 @@
         <v/>
       </c>
       <c r="U149" s="48">
-        <f>M149*P149+K149*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V149" s="37" t="n">
+        <f>M149*P149+K149*V149</f>
+        <v/>
+      </c>
+      <c r="V149" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W149" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -21578,10 +22022,13 @@
         <v/>
       </c>
       <c r="U150" s="48">
-        <f>M150*P150+K150*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V150" s="37" t="n">
+        <f>M150*P150+K150*V150</f>
+        <v/>
+      </c>
+      <c r="V150" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W150" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -21663,10 +22110,13 @@
         <v/>
       </c>
       <c r="U151" s="48">
-        <f>M151*P151+K151*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V151" s="37" t="n">
+        <f>M151*P151+K151*V151</f>
+        <v/>
+      </c>
+      <c r="V151" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W151" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -21748,10 +22198,13 @@
         <v/>
       </c>
       <c r="U152" s="48">
-        <f>M152*P152+K152*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V152" s="37" t="n">
+        <f>M152*P152+K152*V152</f>
+        <v/>
+      </c>
+      <c r="V152" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W152" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -21833,10 +22286,13 @@
         <v/>
       </c>
       <c r="U153" s="48">
-        <f>M153*P153+K153*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V153" s="37" t="n">
+        <f>M153*P153+K153*V153</f>
+        <v/>
+      </c>
+      <c r="V153" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W153" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -21918,10 +22374,13 @@
         <v/>
       </c>
       <c r="U154" s="48">
-        <f>M154*P154+K154*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V154" s="37" t="n">
+        <f>M154*P154+K154*V154</f>
+        <v/>
+      </c>
+      <c r="V154" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W154" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -22003,10 +22462,13 @@
         <v/>
       </c>
       <c r="U155" s="48">
-        <f>M155*P155+K155*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V155" s="37" t="n">
+        <f>M155*P155+K155*V155</f>
+        <v/>
+      </c>
+      <c r="V155" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W155" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -22088,10 +22550,13 @@
         <v/>
       </c>
       <c r="U156" s="48">
-        <f>M156*P156+K156*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V156" s="37" t="n">
+        <f>M156*P156+K156*V156</f>
+        <v/>
+      </c>
+      <c r="V156" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W156" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -22173,10 +22638,13 @@
         <v/>
       </c>
       <c r="U157" s="48">
-        <f>M157*P157+K157*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V157" s="37" t="n">
+        <f>M157*P157+K157*V157</f>
+        <v/>
+      </c>
+      <c r="V157" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W157" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -22258,10 +22726,13 @@
         <v/>
       </c>
       <c r="U158" s="48">
-        <f>M158*P158+K158*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V158" s="37" t="n">
+        <f>M158*P158+K158*V158</f>
+        <v/>
+      </c>
+      <c r="V158" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W158" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -22343,10 +22814,13 @@
         <v/>
       </c>
       <c r="U159" s="48">
-        <f>M159*P159+K159*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V159" s="37" t="n">
+        <f>M159*P159+K159*V159</f>
+        <v/>
+      </c>
+      <c r="V159" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W159" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -22428,10 +22902,13 @@
         <v/>
       </c>
       <c r="U160" s="48">
-        <f>M160*P160+K160*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V160" s="37" t="n">
+        <f>M160*P160+K160*V160</f>
+        <v/>
+      </c>
+      <c r="V160" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W160" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -22513,10 +22990,13 @@
         <v/>
       </c>
       <c r="U161" s="48">
-        <f>M161*P161+K161*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V161" s="37" t="n">
+        <f>M161*P161+K161*V161</f>
+        <v/>
+      </c>
+      <c r="V161" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W161" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -22598,10 +23078,13 @@
         <v/>
       </c>
       <c r="U162" s="48">
-        <f>M162*P162+K162*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V162" s="37" t="n">
+        <f>M162*P162+K162*V162</f>
+        <v/>
+      </c>
+      <c r="V162" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W162" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -22683,10 +23166,13 @@
         <v/>
       </c>
       <c r="U163" s="48">
-        <f>M163*P163+K163*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V163" s="37" t="n">
+        <f>M163*P163+K163*V163</f>
+        <v/>
+      </c>
+      <c r="V163" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W163" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -22768,10 +23254,13 @@
         <v/>
       </c>
       <c r="U164" s="48">
-        <f>M164*P164+K164*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V164" s="37" t="n">
+        <f>M164*P164+K164*V164</f>
+        <v/>
+      </c>
+      <c r="V164" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W164" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -22853,10 +23342,13 @@
         <v/>
       </c>
       <c r="U165" s="48">
-        <f>M165*P165+K165*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V165" s="37" t="n">
+        <f>M165*P165+K165*V165</f>
+        <v/>
+      </c>
+      <c r="V165" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W165" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -22938,10 +23430,13 @@
         <v/>
       </c>
       <c r="U166" s="48">
-        <f>M166*P166+K166*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V166" s="37" t="n">
+        <f>M166*P166+K166*V166</f>
+        <v/>
+      </c>
+      <c r="V166" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W166" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -23023,10 +23518,13 @@
         <v/>
       </c>
       <c r="U167" s="48">
-        <f>M167*P167+K167*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V167" s="37" t="n">
+        <f>M167*P167+K167*V167</f>
+        <v/>
+      </c>
+      <c r="V167" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W167" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -23108,10 +23606,13 @@
         <v/>
       </c>
       <c r="U168" s="48">
-        <f>M168*P168+K168*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V168" s="37" t="n">
+        <f>M168*P168+K168*V168</f>
+        <v/>
+      </c>
+      <c r="V168" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W168" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -23193,10 +23694,13 @@
         <v/>
       </c>
       <c r="U169" s="48">
-        <f>M169*P169+K169*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V169" s="37" t="n">
+        <f>M169*P169+K169*V169</f>
+        <v/>
+      </c>
+      <c r="V169" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W169" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -23278,10 +23782,13 @@
         <v/>
       </c>
       <c r="U170" s="48">
-        <f>M170*P170+K170*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V170" s="37" t="n">
+        <f>M170*P170+K170*V170</f>
+        <v/>
+      </c>
+      <c r="V170" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W170" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -23363,10 +23870,13 @@
         <v/>
       </c>
       <c r="U171" s="48">
-        <f>M171*P171+K171*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V171" s="37" t="n">
+        <f>M171*P171+K171*V171</f>
+        <v/>
+      </c>
+      <c r="V171" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W171" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -23448,10 +23958,13 @@
         <v/>
       </c>
       <c r="U172" s="48">
-        <f>M172*P172+K172*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V172" s="37" t="n">
+        <f>M172*P172+K172*V172</f>
+        <v/>
+      </c>
+      <c r="V172" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W172" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -23533,10 +24046,13 @@
         <v/>
       </c>
       <c r="U173" s="48">
-        <f>M173*P173+K173*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V173" s="37" t="n">
+        <f>M173*P173+K173*V173</f>
+        <v/>
+      </c>
+      <c r="V173" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W173" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -23618,10 +24134,13 @@
         <v/>
       </c>
       <c r="U174" s="48">
-        <f>M174*P174+K174*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V174" s="37" t="n">
+        <f>M174*P174+K174*V174</f>
+        <v/>
+      </c>
+      <c r="V174" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W174" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -23703,10 +24222,13 @@
         <v/>
       </c>
       <c r="U175" s="48">
-        <f>M175*P175+K175*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V175" s="37" t="n">
+        <f>M175*P175+K175*V175</f>
+        <v/>
+      </c>
+      <c r="V175" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W175" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -23788,10 +24310,13 @@
         <v/>
       </c>
       <c r="U176" s="48">
-        <f>M176*P176+K176*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V176" s="37" t="n">
+        <f>M176*P176+K176*V176</f>
+        <v/>
+      </c>
+      <c r="V176" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W176" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -23873,17 +24398,20 @@
         <v/>
       </c>
       <c r="U177" s="48">
-        <f>M177*P177+K177*'01_Cadrage'!$D$30</f>
-        <v/>
-      </c>
-      <c r="V177" s="37" t="n">
+        <f>M177*P177+K177*V177</f>
+        <v/>
+      </c>
+      <c r="V177" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="W177" s="37" t="n">
         <v>2024</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:V2"/>
-    <mergeCell ref="A1:V1"/>
+    <mergeCell ref="A2:W2"/>
+    <mergeCell ref="A1:W1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>